<commit_message>
Add Week 2 Results (Tester)
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2541E5-CD39-4A79-AC10-123395463164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97665B28-7D89-48A3-98EC-AA4FA357AF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1582,6 +1582,12 @@
       <c r="G34" t="s">
         <v>15</v>
       </c>
+      <c r="H34">
+        <v>13</v>
+      </c>
+      <c r="I34">
+        <v>20</v>
+      </c>
       <c r="J34">
         <v>0</v>
       </c>
@@ -1608,6 +1614,12 @@
       <c r="G35" t="s">
         <v>14</v>
       </c>
+      <c r="H35">
+        <v>20</v>
+      </c>
+      <c r="I35">
+        <v>13</v>
+      </c>
       <c r="J35">
         <v>0</v>
       </c>
@@ -1634,6 +1646,12 @@
       <c r="G36" t="s">
         <v>15</v>
       </c>
+      <c r="H36">
+        <v>3</v>
+      </c>
+      <c r="I36">
+        <v>31</v>
+      </c>
       <c r="J36">
         <v>0</v>
       </c>
@@ -1660,6 +1678,12 @@
       <c r="G37" t="s">
         <v>15</v>
       </c>
+      <c r="H37">
+        <v>13</v>
+      </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
       <c r="J37">
         <v>0</v>
       </c>
@@ -1686,6 +1710,12 @@
       <c r="G38" t="s">
         <v>15</v>
       </c>
+      <c r="H38">
+        <v>21</v>
+      </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
       <c r="J38">
         <v>0</v>
       </c>
@@ -1712,6 +1742,12 @@
       <c r="G39" t="s">
         <v>14</v>
       </c>
+      <c r="H39">
+        <v>17</v>
+      </c>
+      <c r="I39">
+        <v>13</v>
+      </c>
       <c r="J39">
         <v>0</v>
       </c>
@@ -1738,6 +1774,12 @@
       <c r="G40" t="s">
         <v>15</v>
       </c>
+      <c r="H40">
+        <v>34</v>
+      </c>
+      <c r="I40">
+        <v>31</v>
+      </c>
       <c r="J40">
         <v>0</v>
       </c>
@@ -1764,6 +1806,12 @@
       <c r="G41" t="s">
         <v>14</v>
       </c>
+      <c r="H41">
+        <v>17</v>
+      </c>
+      <c r="I41">
+        <v>31</v>
+      </c>
       <c r="J41">
         <v>0</v>
       </c>
@@ -1790,6 +1838,12 @@
       <c r="G42" t="s">
         <v>14</v>
       </c>
+      <c r="H42">
+        <v>12</v>
+      </c>
+      <c r="I42">
+        <v>15</v>
+      </c>
       <c r="J42">
         <v>0</v>
       </c>
@@ -1816,6 +1870,12 @@
       <c r="G43" t="s">
         <v>15</v>
       </c>
+      <c r="H43">
+        <v>27</v>
+      </c>
+      <c r="I43">
+        <v>17</v>
+      </c>
       <c r="J43">
         <v>0</v>
       </c>
@@ -1842,6 +1902,12 @@
       <c r="G44" t="s">
         <v>15</v>
       </c>
+      <c r="H44">
+        <v>14</v>
+      </c>
+      <c r="I44">
+        <v>24</v>
+      </c>
       <c r="J44">
         <v>0</v>
       </c>
@@ -1868,6 +1934,12 @@
       <c r="G45" t="s">
         <v>14</v>
       </c>
+      <c r="H45">
+        <v>31</v>
+      </c>
+      <c r="I45">
+        <v>12</v>
+      </c>
       <c r="J45">
         <v>0</v>
       </c>
@@ -1894,6 +1966,12 @@
       <c r="G46" t="s">
         <v>15</v>
       </c>
+      <c r="H46">
+        <v>31</v>
+      </c>
+      <c r="I46">
+        <v>17</v>
+      </c>
       <c r="J46">
         <v>0</v>
       </c>
@@ -1920,6 +1998,12 @@
       <c r="G47" t="s">
         <v>14</v>
       </c>
+      <c r="H47">
+        <v>14</v>
+      </c>
+      <c r="I47">
+        <v>31</v>
+      </c>
       <c r="J47">
         <v>0</v>
       </c>
@@ -1946,6 +2030,12 @@
       <c r="G48" t="s">
         <v>14</v>
       </c>
+      <c r="H48">
+        <v>24</v>
+      </c>
+      <c r="I48">
+        <v>14</v>
+      </c>
       <c r="J48">
         <v>0</v>
       </c>
@@ -1972,6 +2062,12 @@
       <c r="G49" t="s">
         <v>15</v>
       </c>
+      <c r="H49">
+        <v>31</v>
+      </c>
+      <c r="I49">
+        <v>14</v>
+      </c>
       <c r="J49">
         <v>0</v>
       </c>
@@ -1998,6 +2094,12 @@
       <c r="G50" t="s">
         <v>14</v>
       </c>
+      <c r="H50">
+        <v>10</v>
+      </c>
+      <c r="I50">
+        <v>14</v>
+      </c>
       <c r="J50">
         <v>0</v>
       </c>
@@ -2024,6 +2126,12 @@
       <c r="G51" t="s">
         <v>14</v>
       </c>
+      <c r="H51">
+        <v>31</v>
+      </c>
+      <c r="I51">
+        <v>34</v>
+      </c>
       <c r="J51">
         <v>0</v>
       </c>
@@ -2050,6 +2158,12 @@
       <c r="G52" t="s">
         <v>15</v>
       </c>
+      <c r="H52">
+        <v>24</v>
+      </c>
+      <c r="I52">
+        <v>17</v>
+      </c>
       <c r="J52">
         <v>0</v>
       </c>
@@ -2076,6 +2190,12 @@
       <c r="G53" t="s">
         <v>14</v>
       </c>
+      <c r="H53">
+        <v>18</v>
+      </c>
+      <c r="I53">
+        <v>21</v>
+      </c>
       <c r="J53">
         <v>0</v>
       </c>
@@ -2102,6 +2222,12 @@
       <c r="G54" t="s">
         <v>15</v>
       </c>
+      <c r="H54">
+        <v>12</v>
+      </c>
+      <c r="I54">
+        <v>31</v>
+      </c>
       <c r="J54">
         <v>0</v>
       </c>
@@ -2128,6 +2254,12 @@
       <c r="G55" t="s">
         <v>14</v>
       </c>
+      <c r="H55">
+        <v>17</v>
+      </c>
+      <c r="I55">
+        <v>35</v>
+      </c>
       <c r="J55">
         <v>0</v>
       </c>
@@ -2154,6 +2286,12 @@
       <c r="G56" t="s">
         <v>14</v>
       </c>
+      <c r="H56">
+        <v>28</v>
+      </c>
+      <c r="I56">
+        <v>10</v>
+      </c>
       <c r="J56">
         <v>0</v>
       </c>
@@ -2180,6 +2318,12 @@
       <c r="G57" t="s">
         <v>14</v>
       </c>
+      <c r="H57">
+        <v>17</v>
+      </c>
+      <c r="I57">
+        <v>24</v>
+      </c>
       <c r="J57">
         <v>0</v>
       </c>
@@ -2206,6 +2350,12 @@
       <c r="G58" t="s">
         <v>15</v>
       </c>
+      <c r="H58">
+        <v>35</v>
+      </c>
+      <c r="I58">
+        <v>17</v>
+      </c>
       <c r="J58">
         <v>0</v>
       </c>
@@ -2232,6 +2382,12 @@
       <c r="G59" t="s">
         <v>14</v>
       </c>
+      <c r="H59">
+        <v>31</v>
+      </c>
+      <c r="I59">
+        <v>3</v>
+      </c>
       <c r="J59">
         <v>0</v>
       </c>
@@ -2258,6 +2414,12 @@
       <c r="G60" t="s">
         <v>15</v>
       </c>
+      <c r="H60">
+        <v>14</v>
+      </c>
+      <c r="I60">
+        <v>10</v>
+      </c>
       <c r="J60">
         <v>0</v>
       </c>
@@ -2284,6 +2446,12 @@
       <c r="G61" t="s">
         <v>15</v>
       </c>
+      <c r="H61">
+        <v>15</v>
+      </c>
+      <c r="I61">
+        <v>12</v>
+      </c>
       <c r="J61">
         <v>0</v>
       </c>
@@ -2310,6 +2478,12 @@
       <c r="G62" t="s">
         <v>15</v>
       </c>
+      <c r="H62">
+        <v>10</v>
+      </c>
+      <c r="I62">
+        <v>28</v>
+      </c>
       <c r="J62">
         <v>0</v>
       </c>
@@ -2336,6 +2510,12 @@
       <c r="G63" t="s">
         <v>14</v>
       </c>
+      <c r="H63">
+        <v>17</v>
+      </c>
+      <c r="I63">
+        <v>27</v>
+      </c>
       <c r="J63">
         <v>0</v>
       </c>
@@ -2362,6 +2542,12 @@
       <c r="G64" t="s">
         <v>14</v>
       </c>
+      <c r="H64">
+        <v>13</v>
+      </c>
+      <c r="I64">
+        <v>24</v>
+      </c>
       <c r="J64">
         <v>0</v>
       </c>
@@ -2387,6 +2573,12 @@
       </c>
       <c r="G65" t="s">
         <v>15</v>
+      </c>
+      <c r="H65">
+        <v>24</v>
+      </c>
+      <c r="I65">
+        <v>13</v>
       </c>
       <c r="J65">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 3 Results (Tester)
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97665B28-7D89-48A3-98EC-AA4FA357AF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78745094-FF35-44DA-A688-91BAF1C6E5FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2606,6 +2606,12 @@
       <c r="G66" t="s">
         <v>14</v>
       </c>
+      <c r="H66">
+        <v>13</v>
+      </c>
+      <c r="I66">
+        <v>27</v>
+      </c>
       <c r="J66">
         <v>0</v>
       </c>
@@ -2632,6 +2638,12 @@
       <c r="G67" t="s">
         <v>15</v>
       </c>
+      <c r="H67">
+        <v>27</v>
+      </c>
+      <c r="I67">
+        <v>13</v>
+      </c>
       <c r="J67">
         <v>0</v>
       </c>
@@ -2658,6 +2670,12 @@
       <c r="G68" t="s">
         <v>14</v>
       </c>
+      <c r="H68">
+        <v>10</v>
+      </c>
+      <c r="I68">
+        <v>38</v>
+      </c>
       <c r="J68">
         <v>0</v>
       </c>
@@ -2684,6 +2702,12 @@
       <c r="G69" t="s">
         <v>14</v>
       </c>
+      <c r="H69">
+        <v>28</v>
+      </c>
+      <c r="I69">
+        <v>20</v>
+      </c>
       <c r="J69">
         <v>0</v>
       </c>
@@ -2710,6 +2734,12 @@
       <c r="G70" t="s">
         <v>15</v>
       </c>
+      <c r="H70">
+        <v>17</v>
+      </c>
+      <c r="I70">
+        <v>24</v>
+      </c>
       <c r="J70">
         <v>0</v>
       </c>
@@ -2736,6 +2766,12 @@
       <c r="G71" t="s">
         <v>14</v>
       </c>
+      <c r="H71">
+        <v>13</v>
+      </c>
+      <c r="I71">
+        <v>14</v>
+      </c>
       <c r="J71">
         <v>0</v>
       </c>
@@ -2762,6 +2798,12 @@
       <c r="G72" t="s">
         <v>14</v>
       </c>
+      <c r="H72">
+        <v>31</v>
+      </c>
+      <c r="I72">
+        <v>17</v>
+      </c>
       <c r="J72">
         <v>0</v>
       </c>
@@ -2788,6 +2830,12 @@
       <c r="G73" t="s">
         <v>15</v>
       </c>
+      <c r="H73">
+        <v>14</v>
+      </c>
+      <c r="I73">
+        <v>13</v>
+      </c>
       <c r="J73">
         <v>0</v>
       </c>
@@ -2814,6 +2862,12 @@
       <c r="G74" t="s">
         <v>15</v>
       </c>
+      <c r="H74">
+        <v>20</v>
+      </c>
+      <c r="I74">
+        <v>28</v>
+      </c>
       <c r="J74">
         <v>0</v>
       </c>
@@ -2840,8 +2894,14 @@
       <c r="G75" t="s">
         <v>15</v>
       </c>
+      <c r="H75">
+        <v>27</v>
+      </c>
+      <c r="I75">
+        <v>21</v>
+      </c>
       <c r="J75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -2866,6 +2926,12 @@
       <c r="G76" t="s">
         <v>15</v>
       </c>
+      <c r="H76">
+        <v>45</v>
+      </c>
+      <c r="I76">
+        <v>7</v>
+      </c>
       <c r="J76">
         <v>0</v>
       </c>
@@ -2892,6 +2958,12 @@
       <c r="G77" t="s">
         <v>14</v>
       </c>
+      <c r="H77">
+        <v>21</v>
+      </c>
+      <c r="I77">
+        <v>24</v>
+      </c>
       <c r="J77">
         <v>0</v>
       </c>
@@ -2918,6 +2990,12 @@
       <c r="G78" t="s">
         <v>15</v>
       </c>
+      <c r="H78">
+        <v>24</v>
+      </c>
+      <c r="I78">
+        <v>21</v>
+      </c>
       <c r="J78">
         <v>0</v>
       </c>
@@ -2944,6 +3022,12 @@
       <c r="G79" t="s">
         <v>15</v>
       </c>
+      <c r="H79">
+        <v>17</v>
+      </c>
+      <c r="I79">
+        <v>20</v>
+      </c>
       <c r="J79">
         <v>0</v>
       </c>
@@ -2970,6 +3054,12 @@
       <c r="G80" t="s">
         <v>14</v>
       </c>
+      <c r="H80">
+        <v>31</v>
+      </c>
+      <c r="I80">
+        <v>8</v>
+      </c>
       <c r="J80">
         <v>0</v>
       </c>
@@ -2996,6 +3086,12 @@
       <c r="G81" t="s">
         <v>15</v>
       </c>
+      <c r="H81">
+        <v>8</v>
+      </c>
+      <c r="I81">
+        <v>31</v>
+      </c>
       <c r="J81">
         <v>0</v>
       </c>
@@ -3022,6 +3118,12 @@
       <c r="G82" t="s">
         <v>14</v>
       </c>
+      <c r="H82">
+        <v>22</v>
+      </c>
+      <c r="I82">
+        <v>25</v>
+      </c>
       <c r="J82">
         <v>0</v>
       </c>
@@ -3048,6 +3150,12 @@
       <c r="G83" t="s">
         <v>14</v>
       </c>
+      <c r="H83">
+        <v>20</v>
+      </c>
+      <c r="I83">
+        <v>17</v>
+      </c>
       <c r="J83">
         <v>0</v>
       </c>
@@ -3074,6 +3182,12 @@
       <c r="G84" t="s">
         <v>15</v>
       </c>
+      <c r="H84">
+        <v>31</v>
+      </c>
+      <c r="I84">
+        <v>35</v>
+      </c>
       <c r="J84">
         <v>0</v>
       </c>
@@ -3100,6 +3214,12 @@
       <c r="G85" t="s">
         <v>15</v>
       </c>
+      <c r="H85">
+        <v>21</v>
+      </c>
+      <c r="I85">
+        <v>17</v>
+      </c>
       <c r="J85">
         <v>0</v>
       </c>
@@ -3126,6 +3246,12 @@
       <c r="G86" t="s">
         <v>14</v>
       </c>
+      <c r="H86">
+        <v>7</v>
+      </c>
+      <c r="I86">
+        <v>45</v>
+      </c>
       <c r="J86">
         <v>0</v>
       </c>
@@ -3152,6 +3278,12 @@
       <c r="G87" t="s">
         <v>14</v>
       </c>
+      <c r="H87">
+        <v>35</v>
+      </c>
+      <c r="I87">
+        <v>31</v>
+      </c>
       <c r="J87">
         <v>0</v>
       </c>
@@ -3178,6 +3310,12 @@
       <c r="G88" t="s">
         <v>15</v>
       </c>
+      <c r="H88">
+        <v>17</v>
+      </c>
+      <c r="I88">
+        <v>31</v>
+      </c>
       <c r="J88">
         <v>0</v>
       </c>
@@ -3204,6 +3342,12 @@
       <c r="G89" t="s">
         <v>14</v>
       </c>
+      <c r="H89">
+        <v>24</v>
+      </c>
+      <c r="I89">
+        <v>17</v>
+      </c>
       <c r="J89">
         <v>0</v>
       </c>
@@ -3230,6 +3374,12 @@
       <c r="G90" t="s">
         <v>14</v>
       </c>
+      <c r="H90">
+        <v>13</v>
+      </c>
+      <c r="I90">
+        <v>20</v>
+      </c>
       <c r="J90">
         <v>0</v>
       </c>
@@ -3256,6 +3406,12 @@
       <c r="G91" t="s">
         <v>15</v>
       </c>
+      <c r="H91">
+        <v>38</v>
+      </c>
+      <c r="I91">
+        <v>10</v>
+      </c>
       <c r="J91">
         <v>0</v>
       </c>
@@ -3282,8 +3438,14 @@
       <c r="G92" t="s">
         <v>14</v>
       </c>
+      <c r="H92">
+        <v>21</v>
+      </c>
+      <c r="I92">
+        <v>27</v>
+      </c>
       <c r="J92">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
@@ -3308,6 +3470,12 @@
       <c r="G93" t="s">
         <v>15</v>
       </c>
+      <c r="H93">
+        <v>25</v>
+      </c>
+      <c r="I93">
+        <v>22</v>
+      </c>
       <c r="J93">
         <v>0</v>
       </c>
@@ -3334,6 +3502,12 @@
       <c r="G94" t="s">
         <v>14</v>
       </c>
+      <c r="H94">
+        <v>17</v>
+      </c>
+      <c r="I94">
+        <v>21</v>
+      </c>
       <c r="J94">
         <v>0</v>
       </c>
@@ -3360,6 +3534,12 @@
       <c r="G95" t="s">
         <v>15</v>
       </c>
+      <c r="H95">
+        <v>20</v>
+      </c>
+      <c r="I95">
+        <v>13</v>
+      </c>
       <c r="J95">
         <v>0</v>
       </c>
@@ -3386,6 +3566,12 @@
       <c r="G96" t="s">
         <v>15</v>
       </c>
+      <c r="H96">
+        <v>35</v>
+      </c>
+      <c r="I96">
+        <v>34</v>
+      </c>
       <c r="J96">
         <v>0</v>
       </c>
@@ -3411,6 +3597,12 @@
       </c>
       <c r="G97" t="s">
         <v>14</v>
+      </c>
+      <c r="H97">
+        <v>34</v>
+      </c>
+      <c r="I97">
+        <v>35</v>
       </c>
       <c r="J97">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 4 Results (Tester)
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78745094-FF35-44DA-A688-91BAF1C6E5FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EA4AC7-F70B-4C0B-89F9-FDF87C124D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3630,8 +3630,14 @@
       <c r="G98" t="s">
         <v>15</v>
       </c>
+      <c r="H98">
+        <v>6</v>
+      </c>
+      <c r="I98">
+        <v>3</v>
+      </c>
       <c r="J98">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
@@ -3656,8 +3662,14 @@
       <c r="G99" t="s">
         <v>14</v>
       </c>
+      <c r="H99">
+        <v>3</v>
+      </c>
+      <c r="I99">
+        <v>6</v>
+      </c>
       <c r="J99">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
@@ -3682,6 +3694,12 @@
       <c r="G100" t="s">
         <v>14</v>
       </c>
+      <c r="H100">
+        <v>21</v>
+      </c>
+      <c r="I100">
+        <v>17</v>
+      </c>
       <c r="J100">
         <v>0</v>
       </c>
@@ -3708,6 +3726,12 @@
       <c r="G101" t="s">
         <v>15</v>
       </c>
+      <c r="H101">
+        <v>27</v>
+      </c>
+      <c r="I101">
+        <v>28</v>
+      </c>
       <c r="J101">
         <v>0</v>
       </c>
@@ -3734,6 +3758,12 @@
       <c r="G102" t="s">
         <v>15</v>
       </c>
+      <c r="H102">
+        <v>31</v>
+      </c>
+      <c r="I102">
+        <v>28</v>
+      </c>
       <c r="J102">
         <v>0</v>
       </c>
@@ -3760,6 +3790,12 @@
       <c r="G103" t="s">
         <v>15</v>
       </c>
+      <c r="H103">
+        <v>17</v>
+      </c>
+      <c r="I103">
+        <v>38</v>
+      </c>
       <c r="J103">
         <v>0</v>
       </c>
@@ -3786,6 +3822,12 @@
       <c r="G104" t="s">
         <v>15</v>
       </c>
+      <c r="H104">
+        <v>21</v>
+      </c>
+      <c r="I104">
+        <v>23</v>
+      </c>
       <c r="J104">
         <v>0</v>
       </c>
@@ -3812,6 +3854,12 @@
       <c r="G105" t="s">
         <v>15</v>
       </c>
+      <c r="H105">
+        <v>28</v>
+      </c>
+      <c r="I105">
+        <v>37</v>
+      </c>
       <c r="J105">
         <v>0</v>
       </c>
@@ -3838,6 +3886,12 @@
       <c r="G106" t="s">
         <v>14</v>
       </c>
+      <c r="H106">
+        <v>21</v>
+      </c>
+      <c r="I106">
+        <v>31</v>
+      </c>
       <c r="J106">
         <v>0</v>
       </c>
@@ -3864,6 +3918,12 @@
       <c r="G107" t="s">
         <v>14</v>
       </c>
+      <c r="H107">
+        <v>28</v>
+      </c>
+      <c r="I107">
+        <v>20</v>
+      </c>
       <c r="J107">
         <v>0</v>
       </c>
@@ -3890,6 +3950,12 @@
       <c r="G108" t="s">
         <v>14</v>
       </c>
+      <c r="H108">
+        <v>38</v>
+      </c>
+      <c r="I108">
+        <v>17</v>
+      </c>
       <c r="J108">
         <v>0</v>
       </c>
@@ -3916,6 +3982,12 @@
       <c r="G109" t="s">
         <v>14</v>
       </c>
+      <c r="H109">
+        <v>35</v>
+      </c>
+      <c r="I109">
+        <v>10</v>
+      </c>
       <c r="J109">
         <v>0</v>
       </c>
@@ -3942,6 +4014,12 @@
       <c r="G110" t="s">
         <v>15</v>
       </c>
+      <c r="H110">
+        <v>31</v>
+      </c>
+      <c r="I110">
+        <v>21</v>
+      </c>
       <c r="J110">
         <v>0</v>
       </c>
@@ -3968,6 +4046,12 @@
       <c r="G111" t="s">
         <v>14</v>
       </c>
+      <c r="H111">
+        <v>20</v>
+      </c>
+      <c r="I111">
+        <v>31</v>
+      </c>
       <c r="J111">
         <v>0</v>
       </c>
@@ -3994,6 +4078,12 @@
       <c r="G112" t="s">
         <v>14</v>
       </c>
+      <c r="H112">
+        <v>37</v>
+      </c>
+      <c r="I112">
+        <v>28</v>
+      </c>
       <c r="J112">
         <v>0</v>
       </c>
@@ -4020,6 +4110,12 @@
       <c r="G113" t="s">
         <v>14</v>
       </c>
+      <c r="H113">
+        <v>24</v>
+      </c>
+      <c r="I113">
+        <v>27</v>
+      </c>
       <c r="J113">
         <v>0</v>
       </c>
@@ -4046,6 +4142,12 @@
       <c r="G114" t="s">
         <v>14</v>
       </c>
+      <c r="H114">
+        <v>13</v>
+      </c>
+      <c r="I114">
+        <v>17</v>
+      </c>
       <c r="J114">
         <v>0</v>
       </c>
@@ -4072,6 +4174,12 @@
       <c r="G115" t="s">
         <v>15</v>
       </c>
+      <c r="H115">
+        <v>17</v>
+      </c>
+      <c r="I115">
+        <v>13</v>
+      </c>
       <c r="J115">
         <v>0</v>
       </c>
@@ -4098,6 +4206,12 @@
       <c r="G116" t="s">
         <v>14</v>
       </c>
+      <c r="H116">
+        <v>28</v>
+      </c>
+      <c r="I116">
+        <v>31</v>
+      </c>
       <c r="J116">
         <v>0</v>
       </c>
@@ -4124,6 +4238,12 @@
       <c r="G117" t="s">
         <v>15</v>
       </c>
+      <c r="H117">
+        <v>17</v>
+      </c>
+      <c r="I117">
+        <v>21</v>
+      </c>
       <c r="J117">
         <v>0</v>
       </c>
@@ -4150,6 +4270,12 @@
       <c r="G118" t="s">
         <v>14</v>
       </c>
+      <c r="H118">
+        <v>23</v>
+      </c>
+      <c r="I118">
+        <v>21</v>
+      </c>
       <c r="J118">
         <v>0</v>
       </c>
@@ -4176,6 +4302,12 @@
       <c r="G119" t="s">
         <v>15</v>
       </c>
+      <c r="H119">
+        <v>27</v>
+      </c>
+      <c r="I119">
+        <v>24</v>
+      </c>
       <c r="J119">
         <v>0</v>
       </c>
@@ -4202,6 +4334,12 @@
       <c r="G120" t="s">
         <v>15</v>
       </c>
+      <c r="H120">
+        <v>20</v>
+      </c>
+      <c r="I120">
+        <v>44</v>
+      </c>
       <c r="J120">
         <v>0</v>
       </c>
@@ -4228,6 +4366,12 @@
       <c r="G121" t="s">
         <v>14</v>
       </c>
+      <c r="H121">
+        <v>31</v>
+      </c>
+      <c r="I121">
+        <v>25</v>
+      </c>
       <c r="J121">
         <v>0</v>
       </c>
@@ -4254,6 +4398,12 @@
       <c r="G122" t="s">
         <v>15</v>
       </c>
+      <c r="H122">
+        <v>25</v>
+      </c>
+      <c r="I122">
+        <v>31</v>
+      </c>
       <c r="J122">
         <v>0</v>
       </c>
@@ -4280,6 +4430,12 @@
       <c r="G123" t="s">
         <v>15</v>
       </c>
+      <c r="H123">
+        <v>20</v>
+      </c>
+      <c r="I123">
+        <v>28</v>
+      </c>
       <c r="J123">
         <v>0</v>
       </c>
@@ -4306,6 +4462,12 @@
       <c r="G124" t="s">
         <v>14</v>
       </c>
+      <c r="H124">
+        <v>44</v>
+      </c>
+      <c r="I124">
+        <v>20</v>
+      </c>
       <c r="J124">
         <v>0</v>
       </c>
@@ -4332,6 +4494,12 @@
       <c r="G125" t="s">
         <v>15</v>
       </c>
+      <c r="H125">
+        <v>10</v>
+      </c>
+      <c r="I125">
+        <v>35</v>
+      </c>
       <c r="J125">
         <v>0</v>
       </c>
@@ -4358,6 +4526,12 @@
       <c r="G126" t="s">
         <v>14</v>
       </c>
+      <c r="H126">
+        <v>28</v>
+      </c>
+      <c r="I126">
+        <v>27</v>
+      </c>
       <c r="J126">
         <v>0</v>
       </c>
@@ -4384,6 +4558,12 @@
       <c r="G127" t="s">
         <v>15</v>
       </c>
+      <c r="H127">
+        <v>31</v>
+      </c>
+      <c r="I127">
+        <v>20</v>
+      </c>
       <c r="J127">
         <v>0</v>
       </c>
@@ -4410,8 +4590,14 @@
       <c r="G128" t="s">
         <v>14</v>
       </c>
+      <c r="H128">
+        <v>38</v>
+      </c>
+      <c r="I128">
+        <v>41</v>
+      </c>
       <c r="J128">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -4436,8 +4622,14 @@
       <c r="G129" t="s">
         <v>15</v>
       </c>
+      <c r="H129">
+        <v>41</v>
+      </c>
+      <c r="I129">
+        <v>38</v>
+      </c>
       <c r="J129">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add Week 5 Results (Tester)
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EA4AC7-F70B-4C0B-89F9-FDF87C124D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074802CF-5279-43AD-A7CB-BE8658CE6D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4654,6 +4654,12 @@
       <c r="G130" t="s">
         <v>15</v>
       </c>
+      <c r="H130">
+        <v>27</v>
+      </c>
+      <c r="I130">
+        <v>21</v>
+      </c>
       <c r="J130">
         <v>0</v>
       </c>
@@ -4680,6 +4686,12 @@
       <c r="G131" t="s">
         <v>14</v>
       </c>
+      <c r="H131">
+        <v>21</v>
+      </c>
+      <c r="I131">
+        <v>27</v>
+      </c>
       <c r="J131">
         <v>0</v>
       </c>
@@ -4706,6 +4718,12 @@
       <c r="G132" t="s">
         <v>15</v>
       </c>
+      <c r="H132">
+        <v>17</v>
+      </c>
+      <c r="I132">
+        <v>31</v>
+      </c>
       <c r="J132">
         <v>0</v>
       </c>
@@ -4732,6 +4750,12 @@
       <c r="G133" t="s">
         <v>15</v>
       </c>
+      <c r="H133">
+        <v>15</v>
+      </c>
+      <c r="I133">
+        <v>28</v>
+      </c>
       <c r="J133">
         <v>0</v>
       </c>
@@ -4758,6 +4782,12 @@
       <c r="G134" t="s">
         <v>14</v>
       </c>
+      <c r="H134">
+        <v>28</v>
+      </c>
+      <c r="I134">
+        <v>15</v>
+      </c>
       <c r="J134">
         <v>0</v>
       </c>
@@ -4784,6 +4814,12 @@
       <c r="G135" t="s">
         <v>14</v>
       </c>
+      <c r="H135">
+        <v>21</v>
+      </c>
+      <c r="I135">
+        <v>24</v>
+      </c>
       <c r="J135">
         <v>0</v>
       </c>
@@ -4810,6 +4846,12 @@
       <c r="G136" t="s">
         <v>14</v>
       </c>
+      <c r="H136">
+        <v>31</v>
+      </c>
+      <c r="I136">
+        <v>10</v>
+      </c>
       <c r="J136">
         <v>0</v>
       </c>
@@ -4836,6 +4878,12 @@
       <c r="G137" t="s">
         <v>14</v>
       </c>
+      <c r="H137">
+        <v>3</v>
+      </c>
+      <c r="I137">
+        <v>28</v>
+      </c>
       <c r="J137">
         <v>0</v>
       </c>
@@ -4862,6 +4910,12 @@
       <c r="G138" t="s">
         <v>14</v>
       </c>
+      <c r="H138">
+        <v>31</v>
+      </c>
+      <c r="I138">
+        <v>27</v>
+      </c>
       <c r="J138">
         <v>0</v>
       </c>
@@ -4888,6 +4942,12 @@
       <c r="G139" t="s">
         <v>14</v>
       </c>
+      <c r="H139">
+        <v>31</v>
+      </c>
+      <c r="I139">
+        <v>17</v>
+      </c>
       <c r="J139">
         <v>0</v>
       </c>
@@ -4914,6 +4974,12 @@
       <c r="G140" t="s">
         <v>15</v>
       </c>
+      <c r="H140">
+        <v>24</v>
+      </c>
+      <c r="I140">
+        <v>21</v>
+      </c>
       <c r="J140">
         <v>0</v>
       </c>
@@ -4940,6 +5006,12 @@
       <c r="G141" t="s">
         <v>14</v>
       </c>
+      <c r="H141">
+        <v>20</v>
+      </c>
+      <c r="I141">
+        <v>27</v>
+      </c>
       <c r="J141">
         <v>0</v>
       </c>
@@ -4966,6 +5038,12 @@
       <c r="G142" t="s">
         <v>14</v>
       </c>
+      <c r="H142">
+        <v>13</v>
+      </c>
+      <c r="I142">
+        <v>16</v>
+      </c>
       <c r="J142">
         <v>0</v>
       </c>
@@ -4992,6 +5070,12 @@
       <c r="G143" t="s">
         <v>15</v>
       </c>
+      <c r="H143">
+        <v>21</v>
+      </c>
+      <c r="I143">
+        <v>25</v>
+      </c>
       <c r="J143">
         <v>0</v>
       </c>
@@ -5018,6 +5102,12 @@
       <c r="G144" t="s">
         <v>15</v>
       </c>
+      <c r="H144">
+        <v>10</v>
+      </c>
+      <c r="I144">
+        <v>31</v>
+      </c>
       <c r="J144">
         <v>0</v>
       </c>
@@ -5044,6 +5134,12 @@
       <c r="G145" t="s">
         <v>14</v>
       </c>
+      <c r="H145">
+        <v>12</v>
+      </c>
+      <c r="I145">
+        <v>15</v>
+      </c>
       <c r="J145">
         <v>0</v>
       </c>
@@ -5070,6 +5166,12 @@
       <c r="G146" t="s">
         <v>15</v>
       </c>
+      <c r="H146">
+        <v>27</v>
+      </c>
+      <c r="I146">
+        <v>28</v>
+      </c>
       <c r="J146">
         <v>0</v>
       </c>
@@ -5096,6 +5198,12 @@
       <c r="G147" t="s">
         <v>15</v>
       </c>
+      <c r="H147">
+        <v>15</v>
+      </c>
+      <c r="I147">
+        <v>12</v>
+      </c>
       <c r="J147">
         <v>0</v>
       </c>
@@ -5122,6 +5230,12 @@
       <c r="G148" t="s">
         <v>14</v>
       </c>
+      <c r="H148">
+        <v>13</v>
+      </c>
+      <c r="I148">
+        <v>18</v>
+      </c>
       <c r="J148">
         <v>0</v>
       </c>
@@ -5148,6 +5262,12 @@
       <c r="G149" t="s">
         <v>15</v>
       </c>
+      <c r="H149">
+        <v>28</v>
+      </c>
+      <c r="I149">
+        <v>3</v>
+      </c>
       <c r="J149">
         <v>0</v>
       </c>
@@ -5174,6 +5294,12 @@
       <c r="G150" t="s">
         <v>14</v>
       </c>
+      <c r="H150">
+        <v>28</v>
+      </c>
+      <c r="I150">
+        <v>27</v>
+      </c>
       <c r="J150">
         <v>0</v>
       </c>
@@ -5200,6 +5326,12 @@
       <c r="G151" t="s">
         <v>14</v>
       </c>
+      <c r="H151">
+        <v>25</v>
+      </c>
+      <c r="I151">
+        <v>21</v>
+      </c>
       <c r="J151">
         <v>0</v>
       </c>
@@ -5226,6 +5358,12 @@
       <c r="G152" t="s">
         <v>15</v>
       </c>
+      <c r="H152">
+        <v>16</v>
+      </c>
+      <c r="I152">
+        <v>13</v>
+      </c>
       <c r="J152">
         <v>0</v>
       </c>
@@ -5252,6 +5390,12 @@
       <c r="G153" t="s">
         <v>15</v>
       </c>
+      <c r="H153">
+        <v>27</v>
+      </c>
+      <c r="I153">
+        <v>31</v>
+      </c>
       <c r="J153">
         <v>0</v>
       </c>
@@ -5278,6 +5422,12 @@
       <c r="G154" t="s">
         <v>15</v>
       </c>
+      <c r="H154">
+        <v>17</v>
+      </c>
+      <c r="I154">
+        <v>20</v>
+      </c>
       <c r="J154">
         <v>0</v>
       </c>
@@ -5304,6 +5454,12 @@
       <c r="G155" t="s">
         <v>14</v>
       </c>
+      <c r="H155">
+        <v>20</v>
+      </c>
+      <c r="I155">
+        <v>17</v>
+      </c>
       <c r="J155">
         <v>0</v>
       </c>
@@ -5330,6 +5486,12 @@
       <c r="G156" t="s">
         <v>15</v>
       </c>
+      <c r="H156">
+        <v>27</v>
+      </c>
+      <c r="I156">
+        <v>20</v>
+      </c>
       <c r="J156">
         <v>0</v>
       </c>
@@ -5356,6 +5518,12 @@
       <c r="G157" t="s">
         <v>15</v>
       </c>
+      <c r="H157">
+        <v>18</v>
+      </c>
+      <c r="I157">
+        <v>13</v>
+      </c>
       <c r="J157">
         <v>0</v>
       </c>
@@ -5382,6 +5550,12 @@
       <c r="G158" t="s">
         <v>14</v>
       </c>
+      <c r="H158">
+        <v>16</v>
+      </c>
+      <c r="I158">
+        <v>21</v>
+      </c>
       <c r="J158">
         <v>0</v>
       </c>
@@ -5407,6 +5581,12 @@
       </c>
       <c r="G159" t="s">
         <v>15</v>
+      </c>
+      <c r="H159">
+        <v>21</v>
+      </c>
+      <c r="I159">
+        <v>16</v>
       </c>
       <c r="J159">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 1 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B5F7E3-1282-40DD-8807-9FB53F55BDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E099A462-C317-4D9E-8E24-488FBE7DB6A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -558,6 +558,12 @@
       <c r="G2" t="s">
         <v>14</v>
       </c>
+      <c r="H2">
+        <v>13</v>
+      </c>
+      <c r="I2">
+        <v>24</v>
+      </c>
       <c r="J2">
         <v>0</v>
       </c>
@@ -584,6 +590,12 @@
       <c r="G3" t="s">
         <v>15</v>
       </c>
+      <c r="H3">
+        <v>24</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
       <c r="J3">
         <v>0</v>
       </c>
@@ -610,8 +622,14 @@
       <c r="G4" t="s">
         <v>14</v>
       </c>
+      <c r="H4">
+        <v>27</v>
+      </c>
+      <c r="I4">
+        <v>24</v>
+      </c>
       <c r="J4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -636,8 +654,14 @@
       <c r="G5" t="s">
         <v>15</v>
       </c>
+      <c r="H5">
+        <v>24</v>
+      </c>
+      <c r="I5">
+        <v>27</v>
+      </c>
       <c r="J5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -662,6 +686,12 @@
       <c r="G6" t="s">
         <v>14</v>
       </c>
+      <c r="H6">
+        <v>7</v>
+      </c>
+      <c r="I6">
+        <v>19</v>
+      </c>
       <c r="J6">
         <v>0</v>
       </c>
@@ -688,6 +718,12 @@
       <c r="G7" t="s">
         <v>14</v>
       </c>
+      <c r="H7">
+        <v>20</v>
+      </c>
+      <c r="I7">
+        <v>17</v>
+      </c>
       <c r="J7">
         <v>0</v>
       </c>
@@ -714,6 +750,12 @@
       <c r="G8" t="s">
         <v>14</v>
       </c>
+      <c r="H8">
+        <v>31</v>
+      </c>
+      <c r="I8">
+        <v>35</v>
+      </c>
       <c r="J8">
         <v>0</v>
       </c>
@@ -740,6 +782,12 @@
       <c r="G9" t="s">
         <v>14</v>
       </c>
+      <c r="H9">
+        <v>27</v>
+      </c>
+      <c r="I9">
+        <v>31</v>
+      </c>
       <c r="J9">
         <v>0</v>
       </c>
@@ -766,6 +814,12 @@
       <c r="G10" t="s">
         <v>15</v>
       </c>
+      <c r="H10">
+        <v>13</v>
+      </c>
+      <c r="I10">
+        <v>31</v>
+      </c>
       <c r="J10">
         <v>0</v>
       </c>
@@ -792,6 +846,12 @@
       <c r="G11" t="s">
         <v>14</v>
       </c>
+      <c r="H11">
+        <v>31</v>
+      </c>
+      <c r="I11">
+        <v>13</v>
+      </c>
       <c r="J11">
         <v>0</v>
       </c>
@@ -818,8 +878,14 @@
       <c r="G12" t="s">
         <v>15</v>
       </c>
+      <c r="H12">
+        <v>22</v>
+      </c>
+      <c r="I12">
+        <v>10</v>
+      </c>
       <c r="J12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -844,6 +910,12 @@
       <c r="G13" t="s">
         <v>14</v>
       </c>
+      <c r="H13">
+        <v>7</v>
+      </c>
+      <c r="I13">
+        <v>19</v>
+      </c>
       <c r="J13">
         <v>0</v>
       </c>
@@ -870,6 +942,12 @@
       <c r="G14" t="s">
         <v>14</v>
       </c>
+      <c r="H14">
+        <v>31</v>
+      </c>
+      <c r="I14">
+        <v>21</v>
+      </c>
       <c r="J14">
         <v>0</v>
       </c>
@@ -896,6 +974,12 @@
       <c r="G15" t="s">
         <v>15</v>
       </c>
+      <c r="H15">
+        <v>35</v>
+      </c>
+      <c r="I15">
+        <v>7</v>
+      </c>
       <c r="J15">
         <v>0</v>
       </c>
@@ -922,6 +1006,12 @@
       <c r="G16" t="s">
         <v>14</v>
       </c>
+      <c r="H16">
+        <v>20</v>
+      </c>
+      <c r="I16">
+        <v>21</v>
+      </c>
       <c r="J16">
         <v>0</v>
       </c>
@@ -948,6 +1038,12 @@
       <c r="G17" t="s">
         <v>15</v>
       </c>
+      <c r="H17">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>27</v>
+      </c>
       <c r="J17">
         <v>0</v>
       </c>
@@ -974,6 +1070,12 @@
       <c r="G18" t="s">
         <v>15</v>
       </c>
+      <c r="H18">
+        <v>35</v>
+      </c>
+      <c r="I18">
+        <v>31</v>
+      </c>
       <c r="J18">
         <v>0</v>
       </c>
@@ -1000,6 +1102,12 @@
       <c r="G19" t="s">
         <v>15</v>
       </c>
+      <c r="H19">
+        <v>19</v>
+      </c>
+      <c r="I19">
+        <v>7</v>
+      </c>
       <c r="J19">
         <v>0</v>
       </c>
@@ -1026,6 +1134,12 @@
       <c r="G20" t="s">
         <v>14</v>
       </c>
+      <c r="H20">
+        <v>10</v>
+      </c>
+      <c r="I20">
+        <v>13</v>
+      </c>
       <c r="J20">
         <v>0</v>
       </c>
@@ -1052,6 +1166,12 @@
       <c r="G21" t="s">
         <v>15</v>
       </c>
+      <c r="H21">
+        <v>21</v>
+      </c>
+      <c r="I21">
+        <v>20</v>
+      </c>
       <c r="J21">
         <v>0</v>
       </c>
@@ -1078,6 +1198,12 @@
       <c r="G22" t="s">
         <v>14</v>
       </c>
+      <c r="H22">
+        <v>7</v>
+      </c>
+      <c r="I22">
+        <v>35</v>
+      </c>
       <c r="J22">
         <v>0</v>
       </c>
@@ -1104,6 +1230,12 @@
       <c r="G23" t="s">
         <v>15</v>
       </c>
+      <c r="H23">
+        <v>21</v>
+      </c>
+      <c r="I23">
+        <v>31</v>
+      </c>
       <c r="J23">
         <v>0</v>
       </c>
@@ -1130,6 +1262,12 @@
       <c r="G24" t="s">
         <v>14</v>
       </c>
+      <c r="H24">
+        <v>13</v>
+      </c>
+      <c r="I24">
+        <v>16</v>
+      </c>
       <c r="J24">
         <v>0</v>
       </c>
@@ -1156,6 +1294,12 @@
       <c r="G25" t="s">
         <v>15</v>
       </c>
+      <c r="H25">
+        <v>13</v>
+      </c>
+      <c r="I25">
+        <v>10</v>
+      </c>
       <c r="J25">
         <v>0</v>
       </c>
@@ -1182,6 +1326,12 @@
       <c r="G26" t="s">
         <v>15</v>
       </c>
+      <c r="H26">
+        <v>27</v>
+      </c>
+      <c r="I26">
+        <v>20</v>
+      </c>
       <c r="J26">
         <v>0</v>
       </c>
@@ -1208,6 +1358,12 @@
       <c r="G27" t="s">
         <v>15</v>
       </c>
+      <c r="H27">
+        <v>17</v>
+      </c>
+      <c r="I27">
+        <v>20</v>
+      </c>
       <c r="J27">
         <v>0</v>
       </c>
@@ -1234,6 +1390,12 @@
       <c r="G28" t="s">
         <v>15</v>
       </c>
+      <c r="H28">
+        <v>19</v>
+      </c>
+      <c r="I28">
+        <v>7</v>
+      </c>
       <c r="J28">
         <v>0</v>
       </c>
@@ -1260,8 +1422,14 @@
       <c r="G29" t="s">
         <v>14</v>
       </c>
+      <c r="H29">
+        <v>10</v>
+      </c>
+      <c r="I29">
+        <v>22</v>
+      </c>
       <c r="J29">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -1286,6 +1454,12 @@
       <c r="G30" t="s">
         <v>15</v>
       </c>
+      <c r="H30">
+        <v>16</v>
+      </c>
+      <c r="I30">
+        <v>13</v>
+      </c>
       <c r="J30">
         <v>0</v>
       </c>
@@ -1312,6 +1486,12 @@
       <c r="G31" t="s">
         <v>14</v>
       </c>
+      <c r="H31">
+        <v>20</v>
+      </c>
+      <c r="I31">
+        <v>27</v>
+      </c>
       <c r="J31">
         <v>0</v>
       </c>
@@ -1338,6 +1518,12 @@
       <c r="G32" t="s">
         <v>14</v>
       </c>
+      <c r="H32">
+        <v>21</v>
+      </c>
+      <c r="I32">
+        <v>35</v>
+      </c>
       <c r="J32">
         <v>0</v>
       </c>
@@ -1364,6 +1550,12 @@
       <c r="G33" t="s">
         <v>15</v>
       </c>
+      <c r="H33">
+        <v>35</v>
+      </c>
+      <c r="I33">
+        <v>21</v>
+      </c>
       <c r="J33">
         <v>0</v>
       </c>
@@ -2457,7 +2649,7 @@
         <v>15</v>
       </c>
       <c r="J75">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -2899,7 +3091,7 @@
         <v>14</v>
       </c>
       <c r="J92">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
@@ -3055,7 +3247,7 @@
         <v>15</v>
       </c>
       <c r="J98">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
@@ -3081,7 +3273,7 @@
         <v>14</v>
       </c>
       <c r="J99">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
@@ -3835,7 +4027,7 @@
         <v>14</v>
       </c>
       <c r="J128">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -3861,7 +4053,7 @@
         <v>15</v>
       </c>
       <c r="J129">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
@@ -4901,7 +5093,7 @@
         <v>14</v>
       </c>
       <c r="J169">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
@@ -4927,7 +5119,7 @@
         <v>15</v>
       </c>
       <c r="J170">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.35">
@@ -5343,7 +5535,7 @@
         <v>15</v>
       </c>
       <c r="J186">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.35">
@@ -5369,7 +5561,7 @@
         <v>14</v>
       </c>
       <c r="J187">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add Week 2 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E099A462-C317-4D9E-8E24-488FBE7DB6A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3C6E21-6816-43E9-BEB4-F2C22413A747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1582,6 +1582,12 @@
       <c r="G34" t="s">
         <v>15</v>
       </c>
+      <c r="H34">
+        <v>33</v>
+      </c>
+      <c r="I34">
+        <v>30</v>
+      </c>
       <c r="J34">
         <v>0</v>
       </c>
@@ -1608,6 +1614,12 @@
       <c r="G35" t="s">
         <v>14</v>
       </c>
+      <c r="H35">
+        <v>30</v>
+      </c>
+      <c r="I35">
+        <v>33</v>
+      </c>
       <c r="J35">
         <v>0</v>
       </c>
@@ -1634,6 +1646,12 @@
       <c r="G36" t="s">
         <v>15</v>
       </c>
+      <c r="H36">
+        <v>9</v>
+      </c>
+      <c r="I36">
+        <v>15</v>
+      </c>
       <c r="J36">
         <v>0</v>
       </c>
@@ -1660,8 +1678,14 @@
       <c r="G37" t="s">
         <v>15</v>
       </c>
+      <c r="H37">
+        <v>10</v>
+      </c>
+      <c r="I37">
+        <v>13</v>
+      </c>
       <c r="J37">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
@@ -1686,6 +1710,12 @@
       <c r="G38" t="s">
         <v>15</v>
       </c>
+      <c r="H38">
+        <v>28</v>
+      </c>
+      <c r="I38">
+        <v>17</v>
+      </c>
       <c r="J38">
         <v>0</v>
       </c>
@@ -1712,8 +1742,14 @@
       <c r="G39" t="s">
         <v>14</v>
       </c>
+      <c r="H39">
+        <v>13</v>
+      </c>
+      <c r="I39">
+        <v>10</v>
+      </c>
       <c r="J39">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
@@ -1738,6 +1774,12 @@
       <c r="G40" t="s">
         <v>15</v>
       </c>
+      <c r="H40">
+        <v>27</v>
+      </c>
+      <c r="I40">
+        <v>24</v>
+      </c>
       <c r="J40">
         <v>0</v>
       </c>
@@ -1764,6 +1806,12 @@
       <c r="G41" t="s">
         <v>14</v>
       </c>
+      <c r="H41">
+        <v>23</v>
+      </c>
+      <c r="I41">
+        <v>26</v>
+      </c>
       <c r="J41">
         <v>0</v>
       </c>
@@ -1790,6 +1838,12 @@
       <c r="G42" t="s">
         <v>14</v>
       </c>
+      <c r="H42">
+        <v>13</v>
+      </c>
+      <c r="I42">
+        <v>31</v>
+      </c>
       <c r="J42">
         <v>0</v>
       </c>
@@ -1816,6 +1870,12 @@
       <c r="G43" t="s">
         <v>15</v>
       </c>
+      <c r="H43">
+        <v>42</v>
+      </c>
+      <c r="I43">
+        <v>38</v>
+      </c>
       <c r="J43">
         <v>0</v>
       </c>
@@ -1842,6 +1902,12 @@
       <c r="G44" t="s">
         <v>15</v>
       </c>
+      <c r="H44">
+        <v>16</v>
+      </c>
+      <c r="I44">
+        <v>14</v>
+      </c>
       <c r="J44">
         <v>0</v>
       </c>
@@ -1868,6 +1934,12 @@
       <c r="G45" t="s">
         <v>14</v>
       </c>
+      <c r="H45">
+        <v>35</v>
+      </c>
+      <c r="I45">
+        <v>10</v>
+      </c>
       <c r="J45">
         <v>0</v>
       </c>
@@ -1894,6 +1966,12 @@
       <c r="G46" t="s">
         <v>15</v>
       </c>
+      <c r="H46">
+        <v>26</v>
+      </c>
+      <c r="I46">
+        <v>23</v>
+      </c>
       <c r="J46">
         <v>0</v>
       </c>
@@ -1920,6 +1998,12 @@
       <c r="G47" t="s">
         <v>14</v>
       </c>
+      <c r="H47">
+        <v>21</v>
+      </c>
+      <c r="I47">
+        <v>35</v>
+      </c>
       <c r="J47">
         <v>0</v>
       </c>
@@ -1946,6 +2030,12 @@
       <c r="G48" t="s">
         <v>14</v>
       </c>
+      <c r="H48">
+        <v>14</v>
+      </c>
+      <c r="I48">
+        <v>16</v>
+      </c>
       <c r="J48">
         <v>0</v>
       </c>
@@ -1972,6 +2062,12 @@
       <c r="G49" t="s">
         <v>15</v>
       </c>
+      <c r="H49">
+        <v>35</v>
+      </c>
+      <c r="I49">
+        <v>21</v>
+      </c>
       <c r="J49">
         <v>0</v>
       </c>
@@ -1998,6 +2094,12 @@
       <c r="G50" t="s">
         <v>14</v>
       </c>
+      <c r="H50">
+        <v>3</v>
+      </c>
+      <c r="I50">
+        <v>42</v>
+      </c>
       <c r="J50">
         <v>0</v>
       </c>
@@ -2024,6 +2126,12 @@
       <c r="G51" t="s">
         <v>14</v>
       </c>
+      <c r="H51">
+        <v>24</v>
+      </c>
+      <c r="I51">
+        <v>27</v>
+      </c>
       <c r="J51">
         <v>0</v>
       </c>
@@ -2050,6 +2158,12 @@
       <c r="G52" t="s">
         <v>15</v>
       </c>
+      <c r="H52">
+        <v>20</v>
+      </c>
+      <c r="I52">
+        <v>6</v>
+      </c>
       <c r="J52">
         <v>0</v>
       </c>
@@ -2076,6 +2190,12 @@
       <c r="G53" t="s">
         <v>14</v>
       </c>
+      <c r="H53">
+        <v>17</v>
+      </c>
+      <c r="I53">
+        <v>28</v>
+      </c>
       <c r="J53">
         <v>0</v>
       </c>
@@ -2102,6 +2222,12 @@
       <c r="G54" t="s">
         <v>15</v>
       </c>
+      <c r="H54">
+        <v>10</v>
+      </c>
+      <c r="I54">
+        <v>35</v>
+      </c>
       <c r="J54">
         <v>0</v>
       </c>
@@ -2128,6 +2254,12 @@
       <c r="G55" t="s">
         <v>14</v>
       </c>
+      <c r="H55">
+        <v>10</v>
+      </c>
+      <c r="I55">
+        <v>27</v>
+      </c>
       <c r="J55">
         <v>0</v>
       </c>
@@ -2154,6 +2286,12 @@
       <c r="G56" t="s">
         <v>14</v>
       </c>
+      <c r="H56">
+        <v>17</v>
+      </c>
+      <c r="I56">
+        <v>19</v>
+      </c>
       <c r="J56">
         <v>0</v>
       </c>
@@ -2180,6 +2318,12 @@
       <c r="G57" t="s">
         <v>14</v>
       </c>
+      <c r="H57">
+        <v>6</v>
+      </c>
+      <c r="I57">
+        <v>20</v>
+      </c>
       <c r="J57">
         <v>0</v>
       </c>
@@ -2206,6 +2350,12 @@
       <c r="G58" t="s">
         <v>15</v>
       </c>
+      <c r="H58">
+        <v>27</v>
+      </c>
+      <c r="I58">
+        <v>10</v>
+      </c>
       <c r="J58">
         <v>0</v>
       </c>
@@ -2232,6 +2382,12 @@
       <c r="G59" t="s">
         <v>14</v>
       </c>
+      <c r="H59">
+        <v>15</v>
+      </c>
+      <c r="I59">
+        <v>9</v>
+      </c>
       <c r="J59">
         <v>0</v>
       </c>
@@ -2258,6 +2414,12 @@
       <c r="G60" t="s">
         <v>15</v>
       </c>
+      <c r="H60">
+        <v>42</v>
+      </c>
+      <c r="I60">
+        <v>3</v>
+      </c>
       <c r="J60">
         <v>0</v>
       </c>
@@ -2284,6 +2446,12 @@
       <c r="G61" t="s">
         <v>15</v>
       </c>
+      <c r="H61">
+        <v>31</v>
+      </c>
+      <c r="I61">
+        <v>13</v>
+      </c>
       <c r="J61">
         <v>0</v>
       </c>
@@ -2310,6 +2478,12 @@
       <c r="G62" t="s">
         <v>15</v>
       </c>
+      <c r="H62">
+        <v>19</v>
+      </c>
+      <c r="I62">
+        <v>17</v>
+      </c>
       <c r="J62">
         <v>0</v>
       </c>
@@ -2336,6 +2510,12 @@
       <c r="G63" t="s">
         <v>14</v>
       </c>
+      <c r="H63">
+        <v>38</v>
+      </c>
+      <c r="I63">
+        <v>42</v>
+      </c>
       <c r="J63">
         <v>0</v>
       </c>
@@ -2362,6 +2542,12 @@
       <c r="G64" t="s">
         <v>14</v>
       </c>
+      <c r="H64">
+        <v>14</v>
+      </c>
+      <c r="I64">
+        <v>27</v>
+      </c>
       <c r="J64">
         <v>0</v>
       </c>
@@ -2387,6 +2573,12 @@
       </c>
       <c r="G65" t="s">
         <v>15</v>
+      </c>
+      <c r="H65">
+        <v>27</v>
+      </c>
+      <c r="I65">
+        <v>14</v>
       </c>
       <c r="J65">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 3 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3C6E21-6816-43E9-BEB4-F2C22413A747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12D6253-E19B-4181-9085-5D26D222419B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2606,6 +2606,12 @@
       <c r="G66" t="s">
         <v>14</v>
       </c>
+      <c r="H66">
+        <v>13</v>
+      </c>
+      <c r="I66">
+        <v>27</v>
+      </c>
       <c r="J66">
         <v>0</v>
       </c>
@@ -2632,6 +2638,12 @@
       <c r="G67" t="s">
         <v>15</v>
       </c>
+      <c r="H67">
+        <v>27</v>
+      </c>
+      <c r="I67">
+        <v>13</v>
+      </c>
       <c r="J67">
         <v>0</v>
       </c>
@@ -2658,6 +2670,12 @@
       <c r="G68" t="s">
         <v>14</v>
       </c>
+      <c r="H68">
+        <v>12</v>
+      </c>
+      <c r="I68">
+        <v>21</v>
+      </c>
       <c r="J68">
         <v>0</v>
       </c>
@@ -2684,6 +2702,12 @@
       <c r="G69" t="s">
         <v>14</v>
       </c>
+      <c r="H69">
+        <v>38</v>
+      </c>
+      <c r="I69">
+        <v>35</v>
+      </c>
       <c r="J69">
         <v>0</v>
       </c>
@@ -2710,6 +2734,12 @@
       <c r="G70" t="s">
         <v>15</v>
       </c>
+      <c r="H70">
+        <v>38</v>
+      </c>
+      <c r="I70">
+        <v>21</v>
+      </c>
       <c r="J70">
         <v>0</v>
       </c>
@@ -2736,6 +2766,12 @@
       <c r="G71" t="s">
         <v>14</v>
       </c>
+      <c r="H71">
+        <v>7</v>
+      </c>
+      <c r="I71">
+        <v>9</v>
+      </c>
       <c r="J71">
         <v>0</v>
       </c>
@@ -2762,6 +2798,12 @@
       <c r="G72" t="s">
         <v>14</v>
       </c>
+      <c r="H72">
+        <v>17</v>
+      </c>
+      <c r="I72">
+        <v>20</v>
+      </c>
       <c r="J72">
         <v>0</v>
       </c>
@@ -2788,6 +2830,12 @@
       <c r="G73" t="s">
         <v>15</v>
       </c>
+      <c r="H73">
+        <v>9</v>
+      </c>
+      <c r="I73">
+        <v>7</v>
+      </c>
       <c r="J73">
         <v>0</v>
       </c>
@@ -2814,6 +2862,12 @@
       <c r="G74" t="s">
         <v>15</v>
       </c>
+      <c r="H74">
+        <v>35</v>
+      </c>
+      <c r="I74">
+        <v>38</v>
+      </c>
       <c r="J74">
         <v>0</v>
       </c>
@@ -2840,6 +2894,12 @@
       <c r="G75" t="s">
         <v>15</v>
       </c>
+      <c r="H75">
+        <v>14</v>
+      </c>
+      <c r="I75">
+        <v>13</v>
+      </c>
       <c r="J75">
         <v>0</v>
       </c>
@@ -2866,6 +2926,12 @@
       <c r="G76" t="s">
         <v>15</v>
       </c>
+      <c r="H76">
+        <v>42</v>
+      </c>
+      <c r="I76">
+        <v>9</v>
+      </c>
       <c r="J76">
         <v>0</v>
       </c>
@@ -2892,6 +2958,12 @@
       <c r="G77" t="s">
         <v>14</v>
       </c>
+      <c r="H77">
+        <v>21</v>
+      </c>
+      <c r="I77">
+        <v>25</v>
+      </c>
       <c r="J77">
         <v>0</v>
       </c>
@@ -2918,6 +2990,12 @@
       <c r="G78" t="s">
         <v>15</v>
       </c>
+      <c r="H78">
+        <v>25</v>
+      </c>
+      <c r="I78">
+        <v>21</v>
+      </c>
       <c r="J78">
         <v>0</v>
       </c>
@@ -2944,6 +3022,12 @@
       <c r="G79" t="s">
         <v>15</v>
       </c>
+      <c r="H79">
+        <v>17</v>
+      </c>
+      <c r="I79">
+        <v>13</v>
+      </c>
       <c r="J79">
         <v>0</v>
       </c>
@@ -2970,6 +3054,12 @@
       <c r="G80" t="s">
         <v>14</v>
       </c>
+      <c r="H80">
+        <v>31</v>
+      </c>
+      <c r="I80">
+        <v>21</v>
+      </c>
       <c r="J80">
         <v>0</v>
       </c>
@@ -2996,6 +3086,12 @@
       <c r="G81" t="s">
         <v>15</v>
       </c>
+      <c r="H81">
+        <v>21</v>
+      </c>
+      <c r="I81">
+        <v>31</v>
+      </c>
       <c r="J81">
         <v>0</v>
       </c>
@@ -3022,6 +3118,12 @@
       <c r="G82" t="s">
         <v>14</v>
       </c>
+      <c r="H82">
+        <v>27</v>
+      </c>
+      <c r="I82">
+        <v>20</v>
+      </c>
       <c r="J82">
         <v>0</v>
       </c>
@@ -3048,6 +3150,12 @@
       <c r="G83" t="s">
         <v>14</v>
       </c>
+      <c r="H83">
+        <v>13</v>
+      </c>
+      <c r="I83">
+        <v>17</v>
+      </c>
       <c r="J83">
         <v>0</v>
       </c>
@@ -3074,6 +3182,12 @@
       <c r="G84" t="s">
         <v>15</v>
       </c>
+      <c r="H84">
+        <v>18</v>
+      </c>
+      <c r="I84">
+        <v>10</v>
+      </c>
       <c r="J84">
         <v>0</v>
       </c>
@@ -3100,6 +3214,12 @@
       <c r="G85" t="s">
         <v>15</v>
       </c>
+      <c r="H85">
+        <v>22</v>
+      </c>
+      <c r="I85">
+        <v>10</v>
+      </c>
       <c r="J85">
         <v>0</v>
       </c>
@@ -3126,6 +3246,12 @@
       <c r="G86" t="s">
         <v>14</v>
       </c>
+      <c r="H86">
+        <v>9</v>
+      </c>
+      <c r="I86">
+        <v>42</v>
+      </c>
       <c r="J86">
         <v>0</v>
       </c>
@@ -3152,6 +3278,12 @@
       <c r="G87" t="s">
         <v>14</v>
       </c>
+      <c r="H87">
+        <v>10</v>
+      </c>
+      <c r="I87">
+        <v>18</v>
+      </c>
       <c r="J87">
         <v>0</v>
       </c>
@@ -3178,6 +3310,12 @@
       <c r="G88" t="s">
         <v>15</v>
       </c>
+      <c r="H88">
+        <v>20</v>
+      </c>
+      <c r="I88">
+        <v>17</v>
+      </c>
       <c r="J88">
         <v>0</v>
       </c>
@@ -3204,6 +3342,12 @@
       <c r="G89" t="s">
         <v>14</v>
       </c>
+      <c r="H89">
+        <v>21</v>
+      </c>
+      <c r="I89">
+        <v>38</v>
+      </c>
       <c r="J89">
         <v>0</v>
       </c>
@@ -3230,6 +3374,12 @@
       <c r="G90" t="s">
         <v>14</v>
       </c>
+      <c r="H90">
+        <v>24</v>
+      </c>
+      <c r="I90">
+        <v>35</v>
+      </c>
       <c r="J90">
         <v>0</v>
       </c>
@@ -3256,6 +3406,12 @@
       <c r="G91" t="s">
         <v>15</v>
       </c>
+      <c r="H91">
+        <v>21</v>
+      </c>
+      <c r="I91">
+        <v>12</v>
+      </c>
       <c r="J91">
         <v>0</v>
       </c>
@@ -3282,6 +3438,12 @@
       <c r="G92" t="s">
         <v>14</v>
       </c>
+      <c r="H92">
+        <v>13</v>
+      </c>
+      <c r="I92">
+        <v>14</v>
+      </c>
       <c r="J92">
         <v>0</v>
       </c>
@@ -3308,6 +3470,12 @@
       <c r="G93" t="s">
         <v>15</v>
       </c>
+      <c r="H93">
+        <v>20</v>
+      </c>
+      <c r="I93">
+        <v>27</v>
+      </c>
       <c r="J93">
         <v>0</v>
       </c>
@@ -3334,6 +3502,12 @@
       <c r="G94" t="s">
         <v>14</v>
       </c>
+      <c r="H94">
+        <v>10</v>
+      </c>
+      <c r="I94">
+        <v>22</v>
+      </c>
       <c r="J94">
         <v>0</v>
       </c>
@@ -3360,6 +3534,12 @@
       <c r="G95" t="s">
         <v>15</v>
       </c>
+      <c r="H95">
+        <v>35</v>
+      </c>
+      <c r="I95">
+        <v>24</v>
+      </c>
       <c r="J95">
         <v>0</v>
       </c>
@@ -3386,6 +3566,12 @@
       <c r="G96" t="s">
         <v>15</v>
       </c>
+      <c r="H96">
+        <v>27</v>
+      </c>
+      <c r="I96">
+        <v>21</v>
+      </c>
       <c r="J96">
         <v>0</v>
       </c>
@@ -3411,6 +3597,12 @@
       </c>
       <c r="G97" t="s">
         <v>14</v>
+      </c>
+      <c r="H97">
+        <v>21</v>
+      </c>
+      <c r="I97">
+        <v>27</v>
       </c>
       <c r="J97">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 4 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12D6253-E19B-4181-9085-5D26D222419B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF4C394-8554-4E1F-97F3-9C513E8CD7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3630,6 +3630,12 @@
       <c r="G98" t="s">
         <v>15</v>
       </c>
+      <c r="H98">
+        <v>7</v>
+      </c>
+      <c r="I98">
+        <v>6</v>
+      </c>
       <c r="J98">
         <v>0</v>
       </c>
@@ -3656,6 +3662,12 @@
       <c r="G99" t="s">
         <v>14</v>
       </c>
+      <c r="H99">
+        <v>6</v>
+      </c>
+      <c r="I99">
+        <v>7</v>
+      </c>
       <c r="J99">
         <v>0</v>
       </c>
@@ -3682,6 +3694,12 @@
       <c r="G100" t="s">
         <v>14</v>
       </c>
+      <c r="H100">
+        <v>14</v>
+      </c>
+      <c r="I100">
+        <v>16</v>
+      </c>
       <c r="J100">
         <v>0</v>
       </c>
@@ -3708,6 +3726,12 @@
       <c r="G101" t="s">
         <v>15</v>
       </c>
+      <c r="H101">
+        <v>21</v>
+      </c>
+      <c r="I101">
+        <v>10</v>
+      </c>
       <c r="J101">
         <v>0</v>
       </c>
@@ -3734,6 +3758,12 @@
       <c r="G102" t="s">
         <v>15</v>
       </c>
+      <c r="H102">
+        <v>21</v>
+      </c>
+      <c r="I102">
+        <v>17</v>
+      </c>
       <c r="J102">
         <v>0</v>
       </c>
@@ -3760,6 +3790,12 @@
       <c r="G103" t="s">
         <v>15</v>
       </c>
+      <c r="H103">
+        <v>10</v>
+      </c>
+      <c r="I103">
+        <v>20</v>
+      </c>
       <c r="J103">
         <v>0</v>
       </c>
@@ -3786,6 +3822,12 @@
       <c r="G104" t="s">
         <v>15</v>
       </c>
+      <c r="H104">
+        <v>28</v>
+      </c>
+      <c r="I104">
+        <v>13</v>
+      </c>
       <c r="J104">
         <v>0</v>
       </c>
@@ -3812,6 +3854,12 @@
       <c r="G105" t="s">
         <v>15</v>
       </c>
+      <c r="H105">
+        <v>22</v>
+      </c>
+      <c r="I105">
+        <v>19</v>
+      </c>
       <c r="J105">
         <v>0</v>
       </c>
@@ -3838,6 +3886,12 @@
       <c r="G106" t="s">
         <v>14</v>
       </c>
+      <c r="H106">
+        <v>20</v>
+      </c>
+      <c r="I106">
+        <v>22</v>
+      </c>
       <c r="J106">
         <v>0</v>
       </c>
@@ -3864,6 +3918,12 @@
       <c r="G107" t="s">
         <v>14</v>
       </c>
+      <c r="H107">
+        <v>18</v>
+      </c>
+      <c r="I107">
+        <v>15</v>
+      </c>
       <c r="J107">
         <v>0</v>
       </c>
@@ -3890,6 +3950,12 @@
       <c r="G108" t="s">
         <v>14</v>
       </c>
+      <c r="H108">
+        <v>20</v>
+      </c>
+      <c r="I108">
+        <v>10</v>
+      </c>
       <c r="J108">
         <v>0</v>
       </c>
@@ -3916,6 +3982,12 @@
       <c r="G109" t="s">
         <v>14</v>
       </c>
+      <c r="H109">
+        <v>21</v>
+      </c>
+      <c r="I109">
+        <v>14</v>
+      </c>
       <c r="J109">
         <v>0</v>
       </c>
@@ -3942,6 +4014,12 @@
       <c r="G110" t="s">
         <v>15</v>
       </c>
+      <c r="H110">
+        <v>22</v>
+      </c>
+      <c r="I110">
+        <v>20</v>
+      </c>
       <c r="J110">
         <v>0</v>
       </c>
@@ -3968,6 +4046,12 @@
       <c r="G111" t="s">
         <v>14</v>
       </c>
+      <c r="H111">
+        <v>13</v>
+      </c>
+      <c r="I111">
+        <v>18</v>
+      </c>
       <c r="J111">
         <v>0</v>
       </c>
@@ -3994,6 +4078,12 @@
       <c r="G112" t="s">
         <v>14</v>
       </c>
+      <c r="H112">
+        <v>19</v>
+      </c>
+      <c r="I112">
+        <v>22</v>
+      </c>
       <c r="J112">
         <v>0</v>
       </c>
@@ -4020,6 +4110,12 @@
       <c r="G113" t="s">
         <v>14</v>
       </c>
+      <c r="H113">
+        <v>17</v>
+      </c>
+      <c r="I113">
+        <v>21</v>
+      </c>
       <c r="J113">
         <v>0</v>
       </c>
@@ -4046,6 +4142,12 @@
       <c r="G114" t="s">
         <v>14</v>
       </c>
+      <c r="H114">
+        <v>18</v>
+      </c>
+      <c r="I114">
+        <v>42</v>
+      </c>
       <c r="J114">
         <v>0</v>
       </c>
@@ -4072,6 +4174,12 @@
       <c r="G115" t="s">
         <v>15</v>
       </c>
+      <c r="H115">
+        <v>42</v>
+      </c>
+      <c r="I115">
+        <v>18</v>
+      </c>
       <c r="J115">
         <v>0</v>
       </c>
@@ -4098,6 +4206,12 @@
       <c r="G116" t="s">
         <v>14</v>
       </c>
+      <c r="H116">
+        <v>17</v>
+      </c>
+      <c r="I116">
+        <v>21</v>
+      </c>
       <c r="J116">
         <v>0</v>
       </c>
@@ -4124,6 +4238,12 @@
       <c r="G117" t="s">
         <v>15</v>
       </c>
+      <c r="H117">
+        <v>16</v>
+      </c>
+      <c r="I117">
+        <v>14</v>
+      </c>
       <c r="J117">
         <v>0</v>
       </c>
@@ -4150,6 +4270,12 @@
       <c r="G118" t="s">
         <v>14</v>
       </c>
+      <c r="H118">
+        <v>13</v>
+      </c>
+      <c r="I118">
+        <v>28</v>
+      </c>
       <c r="J118">
         <v>0</v>
       </c>
@@ -4176,6 +4302,12 @@
       <c r="G119" t="s">
         <v>15</v>
       </c>
+      <c r="H119">
+        <v>21</v>
+      </c>
+      <c r="I119">
+        <v>17</v>
+      </c>
       <c r="J119">
         <v>0</v>
       </c>
@@ -4202,6 +4334,12 @@
       <c r="G120" t="s">
         <v>15</v>
       </c>
+      <c r="H120">
+        <v>29</v>
+      </c>
+      <c r="I120">
+        <v>26</v>
+      </c>
       <c r="J120">
         <v>0</v>
       </c>
@@ -4228,6 +4366,12 @@
       <c r="G121" t="s">
         <v>14</v>
       </c>
+      <c r="H121">
+        <v>21</v>
+      </c>
+      <c r="I121">
+        <v>31</v>
+      </c>
       <c r="J121">
         <v>0</v>
       </c>
@@ -4254,6 +4398,12 @@
       <c r="G122" t="s">
         <v>15</v>
       </c>
+      <c r="H122">
+        <v>31</v>
+      </c>
+      <c r="I122">
+        <v>21</v>
+      </c>
       <c r="J122">
         <v>0</v>
       </c>
@@ -4280,6 +4430,12 @@
       <c r="G123" t="s">
         <v>15</v>
       </c>
+      <c r="H123">
+        <v>15</v>
+      </c>
+      <c r="I123">
+        <v>18</v>
+      </c>
       <c r="J123">
         <v>0</v>
       </c>
@@ -4306,6 +4462,12 @@
       <c r="G124" t="s">
         <v>14</v>
       </c>
+      <c r="H124">
+        <v>26</v>
+      </c>
+      <c r="I124">
+        <v>29</v>
+      </c>
       <c r="J124">
         <v>0</v>
       </c>
@@ -4332,6 +4494,12 @@
       <c r="G125" t="s">
         <v>15</v>
       </c>
+      <c r="H125">
+        <v>14</v>
+      </c>
+      <c r="I125">
+        <v>21</v>
+      </c>
       <c r="J125">
         <v>0</v>
       </c>
@@ -4358,6 +4526,12 @@
       <c r="G126" t="s">
         <v>14</v>
       </c>
+      <c r="H126">
+        <v>10</v>
+      </c>
+      <c r="I126">
+        <v>21</v>
+      </c>
       <c r="J126">
         <v>0</v>
       </c>
@@ -4384,6 +4558,12 @@
       <c r="G127" t="s">
         <v>15</v>
       </c>
+      <c r="H127">
+        <v>18</v>
+      </c>
+      <c r="I127">
+        <v>13</v>
+      </c>
       <c r="J127">
         <v>0</v>
       </c>
@@ -4410,8 +4590,14 @@
       <c r="G128" t="s">
         <v>14</v>
       </c>
+      <c r="H128">
+        <v>21</v>
+      </c>
+      <c r="I128">
+        <v>18</v>
+      </c>
       <c r="J128">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -4436,8 +4622,14 @@
       <c r="G129" t="s">
         <v>15</v>
       </c>
+      <c r="H129">
+        <v>18</v>
+      </c>
+      <c r="I129">
+        <v>21</v>
+      </c>
       <c r="J129">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add Week 5 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF4C394-8554-4E1F-97F3-9C513E8CD7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D306A157-8C07-4A8C-AE92-1DA148666208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4654,6 +4654,12 @@
       <c r="G130" t="s">
         <v>15</v>
       </c>
+      <c r="H130">
+        <v>38</v>
+      </c>
+      <c r="I130">
+        <v>17</v>
+      </c>
       <c r="J130">
         <v>0</v>
       </c>
@@ -4680,6 +4686,12 @@
       <c r="G131" t="s">
         <v>14</v>
       </c>
+      <c r="H131">
+        <v>17</v>
+      </c>
+      <c r="I131">
+        <v>38</v>
+      </c>
       <c r="J131">
         <v>0</v>
       </c>
@@ -4706,6 +4718,12 @@
       <c r="G132" t="s">
         <v>15</v>
       </c>
+      <c r="H132">
+        <v>24</v>
+      </c>
+      <c r="I132">
+        <v>21</v>
+      </c>
       <c r="J132">
         <v>0</v>
       </c>
@@ -4732,6 +4750,12 @@
       <c r="G133" t="s">
         <v>15</v>
       </c>
+      <c r="H133">
+        <v>23</v>
+      </c>
+      <c r="I133">
+        <v>31</v>
+      </c>
       <c r="J133">
         <v>0</v>
       </c>
@@ -4758,6 +4782,12 @@
       <c r="G134" t="s">
         <v>14</v>
       </c>
+      <c r="H134">
+        <v>31</v>
+      </c>
+      <c r="I134">
+        <v>23</v>
+      </c>
       <c r="J134">
         <v>0</v>
       </c>
@@ -4784,6 +4814,12 @@
       <c r="G135" t="s">
         <v>14</v>
       </c>
+      <c r="H135">
+        <v>24</v>
+      </c>
+      <c r="I135">
+        <v>28</v>
+      </c>
       <c r="J135">
         <v>0</v>
       </c>
@@ -4810,6 +4846,12 @@
       <c r="G136" t="s">
         <v>14</v>
       </c>
+      <c r="H136">
+        <v>27</v>
+      </c>
+      <c r="I136">
+        <v>7</v>
+      </c>
       <c r="J136">
         <v>0</v>
       </c>
@@ -4836,6 +4878,12 @@
       <c r="G137" t="s">
         <v>14</v>
       </c>
+      <c r="H137">
+        <v>7</v>
+      </c>
+      <c r="I137">
+        <v>11</v>
+      </c>
       <c r="J137">
         <v>0</v>
       </c>
@@ -4862,6 +4910,12 @@
       <c r="G138" t="s">
         <v>14</v>
       </c>
+      <c r="H138">
+        <v>21</v>
+      </c>
+      <c r="I138">
+        <v>24</v>
+      </c>
       <c r="J138">
         <v>0</v>
       </c>
@@ -4888,6 +4942,12 @@
       <c r="G139" t="s">
         <v>14</v>
       </c>
+      <c r="H139">
+        <v>21</v>
+      </c>
+      <c r="I139">
+        <v>24</v>
+      </c>
       <c r="J139">
         <v>0</v>
       </c>
@@ -4914,6 +4974,12 @@
       <c r="G140" t="s">
         <v>15</v>
       </c>
+      <c r="H140">
+        <v>28</v>
+      </c>
+      <c r="I140">
+        <v>24</v>
+      </c>
       <c r="J140">
         <v>0</v>
       </c>
@@ -4940,6 +5006,12 @@
       <c r="G141" t="s">
         <v>14</v>
       </c>
+      <c r="H141">
+        <v>34</v>
+      </c>
+      <c r="I141">
+        <v>31</v>
+      </c>
       <c r="J141">
         <v>0</v>
       </c>
@@ -4966,6 +5038,12 @@
       <c r="G142" t="s">
         <v>14</v>
       </c>
+      <c r="H142">
+        <v>12</v>
+      </c>
+      <c r="I142">
+        <v>14</v>
+      </c>
       <c r="J142">
         <v>0</v>
       </c>
@@ -4992,6 +5070,12 @@
       <c r="G143" t="s">
         <v>15</v>
       </c>
+      <c r="H143">
+        <v>21</v>
+      </c>
+      <c r="I143">
+        <v>16</v>
+      </c>
       <c r="J143">
         <v>0</v>
       </c>
@@ -5018,6 +5102,12 @@
       <c r="G144" t="s">
         <v>15</v>
       </c>
+      <c r="H144">
+        <v>7</v>
+      </c>
+      <c r="I144">
+        <v>27</v>
+      </c>
       <c r="J144">
         <v>0</v>
       </c>
@@ -5044,6 +5134,12 @@
       <c r="G145" t="s">
         <v>14</v>
       </c>
+      <c r="H145">
+        <v>22</v>
+      </c>
+      <c r="I145">
+        <v>27</v>
+      </c>
       <c r="J145">
         <v>0</v>
       </c>
@@ -5070,6 +5166,12 @@
       <c r="G146" t="s">
         <v>15</v>
       </c>
+      <c r="H146">
+        <v>22</v>
+      </c>
+      <c r="I146">
+        <v>13</v>
+      </c>
       <c r="J146">
         <v>0</v>
       </c>
@@ -5096,6 +5198,12 @@
       <c r="G147" t="s">
         <v>15</v>
       </c>
+      <c r="H147">
+        <v>27</v>
+      </c>
+      <c r="I147">
+        <v>22</v>
+      </c>
       <c r="J147">
         <v>0</v>
       </c>
@@ -5122,6 +5230,12 @@
       <c r="G148" t="s">
         <v>14</v>
       </c>
+      <c r="H148">
+        <v>28</v>
+      </c>
+      <c r="I148">
+        <v>27</v>
+      </c>
       <c r="J148">
         <v>0</v>
       </c>
@@ -5148,6 +5262,12 @@
       <c r="G149" t="s">
         <v>15</v>
       </c>
+      <c r="H149">
+        <v>11</v>
+      </c>
+      <c r="I149">
+        <v>7</v>
+      </c>
       <c r="J149">
         <v>0</v>
       </c>
@@ -5174,6 +5294,12 @@
       <c r="G150" t="s">
         <v>14</v>
       </c>
+      <c r="H150">
+        <v>13</v>
+      </c>
+      <c r="I150">
+        <v>22</v>
+      </c>
       <c r="J150">
         <v>0</v>
       </c>
@@ -5200,6 +5326,12 @@
       <c r="G151" t="s">
         <v>14</v>
       </c>
+      <c r="H151">
+        <v>16</v>
+      </c>
+      <c r="I151">
+        <v>21</v>
+      </c>
       <c r="J151">
         <v>0</v>
       </c>
@@ -5226,6 +5358,12 @@
       <c r="G152" t="s">
         <v>15</v>
       </c>
+      <c r="H152">
+        <v>14</v>
+      </c>
+      <c r="I152">
+        <v>12</v>
+      </c>
       <c r="J152">
         <v>0</v>
       </c>
@@ -5252,6 +5390,12 @@
       <c r="G153" t="s">
         <v>15</v>
       </c>
+      <c r="H153">
+        <v>24</v>
+      </c>
+      <c r="I153">
+        <v>21</v>
+      </c>
       <c r="J153">
         <v>0</v>
       </c>
@@ -5278,6 +5422,12 @@
       <c r="G154" t="s">
         <v>15</v>
       </c>
+      <c r="H154">
+        <v>24</v>
+      </c>
+      <c r="I154">
+        <v>12</v>
+      </c>
       <c r="J154">
         <v>0</v>
       </c>
@@ -5304,6 +5454,12 @@
       <c r="G155" t="s">
         <v>14</v>
       </c>
+      <c r="H155">
+        <v>12</v>
+      </c>
+      <c r="I155">
+        <v>24</v>
+      </c>
       <c r="J155">
         <v>0</v>
       </c>
@@ -5330,6 +5486,12 @@
       <c r="G156" t="s">
         <v>15</v>
       </c>
+      <c r="H156">
+        <v>31</v>
+      </c>
+      <c r="I156">
+        <v>34</v>
+      </c>
       <c r="J156">
         <v>0</v>
       </c>
@@ -5356,6 +5518,12 @@
       <c r="G157" t="s">
         <v>15</v>
       </c>
+      <c r="H157">
+        <v>27</v>
+      </c>
+      <c r="I157">
+        <v>28</v>
+      </c>
       <c r="J157">
         <v>0</v>
       </c>
@@ -5382,6 +5550,12 @@
       <c r="G158" t="s">
         <v>14</v>
       </c>
+      <c r="H158">
+        <v>23</v>
+      </c>
+      <c r="I158">
+        <v>33</v>
+      </c>
       <c r="J158">
         <v>0</v>
       </c>
@@ -5407,6 +5581,12 @@
       </c>
       <c r="G159" t="s">
         <v>15</v>
+      </c>
+      <c r="H159">
+        <v>33</v>
+      </c>
+      <c r="I159">
+        <v>23</v>
       </c>
       <c r="J159">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 6 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D306A157-8C07-4A8C-AE92-1DA148666208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AA7C7F-4309-44EC-8989-1E62C01073FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5614,6 +5614,12 @@
       <c r="G160" t="s">
         <v>15</v>
       </c>
+      <c r="H160">
+        <v>16</v>
+      </c>
+      <c r="I160">
+        <v>13</v>
+      </c>
       <c r="J160">
         <v>0</v>
       </c>
@@ -5640,6 +5646,12 @@
       <c r="G161" t="s">
         <v>14</v>
       </c>
+      <c r="H161">
+        <v>13</v>
+      </c>
+      <c r="I161">
+        <v>16</v>
+      </c>
       <c r="J161">
         <v>0</v>
       </c>
@@ -5666,6 +5678,12 @@
       <c r="G162" t="s">
         <v>14</v>
       </c>
+      <c r="H162">
+        <v>7</v>
+      </c>
+      <c r="I162">
+        <v>24</v>
+      </c>
       <c r="J162">
         <v>0</v>
       </c>
@@ -5692,6 +5710,12 @@
       <c r="G163" t="s">
         <v>15</v>
       </c>
+      <c r="H163">
+        <v>31</v>
+      </c>
+      <c r="I163">
+        <v>27</v>
+      </c>
       <c r="J163">
         <v>0</v>
       </c>
@@ -5718,6 +5742,12 @@
       <c r="G164" t="s">
         <v>14</v>
       </c>
+      <c r="H164">
+        <v>11</v>
+      </c>
+      <c r="I164">
+        <v>14</v>
+      </c>
       <c r="J164">
         <v>0</v>
       </c>
@@ -5744,6 +5774,12 @@
       <c r="G165" t="s">
         <v>14</v>
       </c>
+      <c r="H165">
+        <v>38</v>
+      </c>
+      <c r="I165">
+        <v>17</v>
+      </c>
       <c r="J165">
         <v>0</v>
       </c>
@@ -5770,6 +5806,12 @@
       <c r="G166" t="s">
         <v>14</v>
       </c>
+      <c r="H166">
+        <v>17</v>
+      </c>
+      <c r="I166">
+        <v>21</v>
+      </c>
       <c r="J166">
         <v>0</v>
       </c>
@@ -5796,6 +5838,12 @@
       <c r="G167" t="s">
         <v>14</v>
       </c>
+      <c r="H167">
+        <v>27</v>
+      </c>
+      <c r="I167">
+        <v>31</v>
+      </c>
       <c r="J167">
         <v>0</v>
       </c>
@@ -5822,6 +5870,12 @@
       <c r="G168" t="s">
         <v>15</v>
       </c>
+      <c r="H168">
+        <v>14</v>
+      </c>
+      <c r="I168">
+        <v>11</v>
+      </c>
       <c r="J168">
         <v>0</v>
       </c>
@@ -5848,6 +5902,12 @@
       <c r="G169" t="s">
         <v>14</v>
       </c>
+      <c r="H169">
+        <v>31</v>
+      </c>
+      <c r="I169">
+        <v>34</v>
+      </c>
       <c r="J169">
         <v>0</v>
       </c>
@@ -5874,6 +5934,12 @@
       <c r="G170" t="s">
         <v>15</v>
       </c>
+      <c r="H170">
+        <v>34</v>
+      </c>
+      <c r="I170">
+        <v>31</v>
+      </c>
       <c r="J170">
         <v>0</v>
       </c>
@@ -5900,6 +5966,12 @@
       <c r="G171" t="s">
         <v>14</v>
       </c>
+      <c r="H171">
+        <v>21</v>
+      </c>
+      <c r="I171">
+        <v>23</v>
+      </c>
       <c r="J171">
         <v>0</v>
       </c>
@@ -5926,6 +5998,12 @@
       <c r="G172" t="s">
         <v>15</v>
       </c>
+      <c r="H172">
+        <v>18</v>
+      </c>
+      <c r="I172">
+        <v>15</v>
+      </c>
       <c r="J172">
         <v>0</v>
       </c>
@@ -5952,6 +6030,12 @@
       <c r="G173" t="s">
         <v>15</v>
       </c>
+      <c r="H173">
+        <v>23</v>
+      </c>
+      <c r="I173">
+        <v>21</v>
+      </c>
       <c r="J173">
         <v>0</v>
       </c>
@@ -5978,6 +6062,12 @@
       <c r="G174" t="s">
         <v>15</v>
       </c>
+      <c r="H174">
+        <v>25</v>
+      </c>
+      <c r="I174">
+        <v>28</v>
+      </c>
       <c r="J174">
         <v>0</v>
       </c>
@@ -6004,6 +6094,12 @@
       <c r="G175" t="s">
         <v>15</v>
       </c>
+      <c r="H175">
+        <v>27</v>
+      </c>
+      <c r="I175">
+        <v>20</v>
+      </c>
       <c r="J175">
         <v>0</v>
       </c>
@@ -6030,6 +6126,12 @@
       <c r="G176" t="s">
         <v>14</v>
       </c>
+      <c r="H176">
+        <v>13</v>
+      </c>
+      <c r="I176">
+        <v>24</v>
+      </c>
       <c r="J176">
         <v>0</v>
       </c>
@@ -6056,6 +6158,12 @@
       <c r="G177" t="s">
         <v>15</v>
       </c>
+      <c r="H177">
+        <v>24</v>
+      </c>
+      <c r="I177">
+        <v>13</v>
+      </c>
       <c r="J177">
         <v>0</v>
       </c>
@@ -6082,6 +6190,12 @@
       <c r="G178" t="s">
         <v>14</v>
       </c>
+      <c r="H178">
+        <v>20</v>
+      </c>
+      <c r="I178">
+        <v>27</v>
+      </c>
       <c r="J178">
         <v>0</v>
       </c>
@@ -6108,6 +6222,12 @@
       <c r="G179" t="s">
         <v>15</v>
       </c>
+      <c r="H179">
+        <v>17</v>
+      </c>
+      <c r="I179">
+        <v>38</v>
+      </c>
       <c r="J179">
         <v>0</v>
       </c>
@@ -6134,6 +6254,12 @@
       <c r="G180" t="s">
         <v>15</v>
       </c>
+      <c r="H180">
+        <v>21</v>
+      </c>
+      <c r="I180">
+        <v>17</v>
+      </c>
       <c r="J180">
         <v>0</v>
       </c>
@@ -6160,6 +6286,12 @@
       <c r="G181" t="s">
         <v>14</v>
       </c>
+      <c r="H181">
+        <v>10</v>
+      </c>
+      <c r="I181">
+        <v>13</v>
+      </c>
       <c r="J181">
         <v>0</v>
       </c>
@@ -6186,6 +6318,12 @@
       <c r="G182" t="s">
         <v>14</v>
       </c>
+      <c r="H182">
+        <v>28</v>
+      </c>
+      <c r="I182">
+        <v>25</v>
+      </c>
       <c r="J182">
         <v>0</v>
       </c>
@@ -6212,6 +6350,12 @@
       <c r="G183" t="s">
         <v>15</v>
       </c>
+      <c r="H183">
+        <v>24</v>
+      </c>
+      <c r="I183">
+        <v>7</v>
+      </c>
       <c r="J183">
         <v>0</v>
       </c>
@@ -6238,6 +6382,12 @@
       <c r="G184" t="s">
         <v>15</v>
       </c>
+      <c r="H184">
+        <v>13</v>
+      </c>
+      <c r="I184">
+        <v>10</v>
+      </c>
       <c r="J184">
         <v>0</v>
       </c>
@@ -6264,6 +6414,12 @@
       <c r="G185" t="s">
         <v>14</v>
       </c>
+      <c r="H185">
+        <v>15</v>
+      </c>
+      <c r="I185">
+        <v>18</v>
+      </c>
       <c r="J185">
         <v>0</v>
       </c>
@@ -6290,6 +6446,12 @@
       <c r="G186" t="s">
         <v>15</v>
       </c>
+      <c r="H186">
+        <v>24</v>
+      </c>
+      <c r="I186">
+        <v>31</v>
+      </c>
       <c r="J186">
         <v>0</v>
       </c>
@@ -6315,6 +6477,12 @@
       </c>
       <c r="G187" t="s">
         <v>14</v>
+      </c>
+      <c r="H187">
+        <v>31</v>
+      </c>
+      <c r="I187">
+        <v>24</v>
       </c>
       <c r="J187">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 7 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AA7C7F-4309-44EC-8989-1E62C01073FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868D1197-8BE7-4B59-A0CD-A8533844EB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6510,6 +6510,12 @@
       <c r="G188" t="s">
         <v>15</v>
       </c>
+      <c r="H188">
+        <v>25</v>
+      </c>
+      <c r="I188">
+        <v>23</v>
+      </c>
       <c r="J188">
         <v>0</v>
       </c>
@@ -6536,6 +6542,12 @@
       <c r="G189" t="s">
         <v>14</v>
       </c>
+      <c r="H189">
+        <v>23</v>
+      </c>
+      <c r="I189">
+        <v>25</v>
+      </c>
       <c r="J189">
         <v>0</v>
       </c>
@@ -6562,6 +6574,12 @@
       <c r="G190" t="s">
         <v>15</v>
       </c>
+      <c r="H190">
+        <v>12</v>
+      </c>
+      <c r="I190">
+        <v>15</v>
+      </c>
       <c r="J190">
         <v>0</v>
       </c>
@@ -6588,6 +6606,12 @@
       <c r="G191" t="s">
         <v>15</v>
       </c>
+      <c r="H191">
+        <v>14</v>
+      </c>
+      <c r="I191">
+        <v>27</v>
+      </c>
       <c r="J191">
         <v>0</v>
       </c>
@@ -6614,8 +6638,14 @@
       <c r="G192" t="s">
         <v>15</v>
       </c>
+      <c r="H192">
+        <v>23</v>
+      </c>
+      <c r="I192">
+        <v>23</v>
+      </c>
       <c r="J192">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.35">
@@ -6640,6 +6670,12 @@
       <c r="G193" t="s">
         <v>15</v>
       </c>
+      <c r="H193">
+        <v>14</v>
+      </c>
+      <c r="I193">
+        <v>9</v>
+      </c>
       <c r="J193">
         <v>0</v>
       </c>
@@ -6666,8 +6702,14 @@
       <c r="G194" t="s">
         <v>14</v>
       </c>
+      <c r="H194">
+        <v>23</v>
+      </c>
+      <c r="I194">
+        <v>23</v>
+      </c>
       <c r="J194">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.35">
@@ -6692,6 +6734,12 @@
       <c r="G195" t="s">
         <v>14</v>
       </c>
+      <c r="H195">
+        <v>6</v>
+      </c>
+      <c r="I195">
+        <v>13</v>
+      </c>
       <c r="J195">
         <v>0</v>
       </c>
@@ -6718,6 +6766,12 @@
       <c r="G196" t="s">
         <v>14</v>
       </c>
+      <c r="H196">
+        <v>15</v>
+      </c>
+      <c r="I196">
+        <v>12</v>
+      </c>
       <c r="J196">
         <v>0</v>
       </c>
@@ -6744,6 +6798,12 @@
       <c r="G197" t="s">
         <v>15</v>
       </c>
+      <c r="H197">
+        <v>30</v>
+      </c>
+      <c r="I197">
+        <v>26</v>
+      </c>
       <c r="J197">
         <v>0</v>
       </c>
@@ -6770,6 +6830,12 @@
       <c r="G198" t="s">
         <v>14</v>
       </c>
+      <c r="H198">
+        <v>26</v>
+      </c>
+      <c r="I198">
+        <v>30</v>
+      </c>
       <c r="J198">
         <v>0</v>
       </c>
@@ -6796,6 +6862,12 @@
       <c r="G199" t="s">
         <v>15</v>
       </c>
+      <c r="H199">
+        <v>26</v>
+      </c>
+      <c r="I199">
+        <v>23</v>
+      </c>
       <c r="J199">
         <v>0</v>
       </c>
@@ -6822,6 +6894,12 @@
       <c r="G200" t="s">
         <v>14</v>
       </c>
+      <c r="H200">
+        <v>19</v>
+      </c>
+      <c r="I200">
+        <v>26</v>
+      </c>
       <c r="J200">
         <v>0</v>
       </c>
@@ -6848,6 +6926,12 @@
       <c r="G201" t="s">
         <v>14</v>
       </c>
+      <c r="H201">
+        <v>20</v>
+      </c>
+      <c r="I201">
+        <v>18</v>
+      </c>
       <c r="J201">
         <v>0</v>
       </c>
@@ -6874,8 +6958,14 @@
       <c r="G202" t="s">
         <v>14</v>
       </c>
+      <c r="H202">
+        <v>8</v>
+      </c>
+      <c r="I202">
+        <v>14</v>
+      </c>
       <c r="J202">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.35">
@@ -6900,6 +6990,12 @@
       <c r="G203" t="s">
         <v>15</v>
       </c>
+      <c r="H203">
+        <v>26</v>
+      </c>
+      <c r="I203">
+        <v>19</v>
+      </c>
       <c r="J203">
         <v>0</v>
       </c>
@@ -6926,6 +7022,12 @@
       <c r="G204" t="s">
         <v>15</v>
       </c>
+      <c r="H204">
+        <v>15</v>
+      </c>
+      <c r="I204">
+        <v>14</v>
+      </c>
       <c r="J204">
         <v>0</v>
       </c>
@@ -6952,6 +7054,12 @@
       <c r="G205" t="s">
         <v>14</v>
       </c>
+      <c r="H205">
+        <v>23</v>
+      </c>
+      <c r="I205">
+        <v>26</v>
+      </c>
       <c r="J205">
         <v>0</v>
       </c>
@@ -6978,8 +7086,14 @@
       <c r="G206" t="s">
         <v>15</v>
       </c>
+      <c r="H206">
+        <v>14</v>
+      </c>
+      <c r="I206">
+        <v>8</v>
+      </c>
       <c r="J206">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.35">
@@ -7004,6 +7118,12 @@
       <c r="G207" t="s">
         <v>15</v>
       </c>
+      <c r="H207">
+        <v>19</v>
+      </c>
+      <c r="I207">
+        <v>29</v>
+      </c>
       <c r="J207">
         <v>0</v>
       </c>
@@ -7030,6 +7150,12 @@
       <c r="G208" t="s">
         <v>14</v>
       </c>
+      <c r="H208">
+        <v>14</v>
+      </c>
+      <c r="I208">
+        <v>15</v>
+      </c>
       <c r="J208">
         <v>0</v>
       </c>
@@ -7056,6 +7182,12 @@
       <c r="G209" t="s">
         <v>15</v>
       </c>
+      <c r="H209">
+        <v>18</v>
+      </c>
+      <c r="I209">
+        <v>20</v>
+      </c>
       <c r="J209">
         <v>0</v>
       </c>
@@ -7082,6 +7214,12 @@
       <c r="G210" t="s">
         <v>14</v>
       </c>
+      <c r="H210">
+        <v>27</v>
+      </c>
+      <c r="I210">
+        <v>14</v>
+      </c>
       <c r="J210">
         <v>0</v>
       </c>
@@ -7108,6 +7246,12 @@
       <c r="G211" t="s">
         <v>14</v>
       </c>
+      <c r="H211">
+        <v>29</v>
+      </c>
+      <c r="I211">
+        <v>19</v>
+      </c>
       <c r="J211">
         <v>0</v>
       </c>
@@ -7134,6 +7278,12 @@
       <c r="G212" t="s">
         <v>14</v>
       </c>
+      <c r="H212">
+        <v>9</v>
+      </c>
+      <c r="I212">
+        <v>14</v>
+      </c>
       <c r="J212">
         <v>0</v>
       </c>
@@ -7160,6 +7310,12 @@
       <c r="G213" t="s">
         <v>15</v>
       </c>
+      <c r="H213">
+        <v>13</v>
+      </c>
+      <c r="I213">
+        <v>6</v>
+      </c>
       <c r="J213">
         <v>0</v>
       </c>
@@ -7186,6 +7342,12 @@
       <c r="G214" t="s">
         <v>14</v>
       </c>
+      <c r="H214">
+        <v>34</v>
+      </c>
+      <c r="I214">
+        <v>37</v>
+      </c>
       <c r="J214">
         <v>0</v>
       </c>
@@ -7211,6 +7373,12 @@
       </c>
       <c r="G215" t="s">
         <v>15</v>
+      </c>
+      <c r="H215">
+        <v>37</v>
+      </c>
+      <c r="I215">
+        <v>34</v>
       </c>
       <c r="J215">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 8 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868D1197-8BE7-4B59-A0CD-A8533844EB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B403FC79-FD4F-476A-8C20-1CC885C2C36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7406,6 +7406,12 @@
       <c r="G216" t="s">
         <v>14</v>
       </c>
+      <c r="H216">
+        <v>27</v>
+      </c>
+      <c r="I216">
+        <v>28</v>
+      </c>
       <c r="J216">
         <v>0</v>
       </c>
@@ -7432,6 +7438,12 @@
       <c r="G217" t="s">
         <v>15</v>
       </c>
+      <c r="H217">
+        <v>28</v>
+      </c>
+      <c r="I217">
+        <v>27</v>
+      </c>
       <c r="J217">
         <v>0</v>
       </c>
@@ -7458,6 +7470,12 @@
       <c r="G218" t="s">
         <v>14</v>
       </c>
+      <c r="H218">
+        <v>12</v>
+      </c>
+      <c r="I218">
+        <v>20</v>
+      </c>
       <c r="J218">
         <v>0</v>
       </c>
@@ -7484,6 +7502,12 @@
       <c r="G219" t="s">
         <v>14</v>
       </c>
+      <c r="H219">
+        <v>17</v>
+      </c>
+      <c r="I219">
+        <v>24</v>
+      </c>
       <c r="J219">
         <v>0</v>
       </c>
@@ -7510,6 +7534,12 @@
       <c r="G220" t="s">
         <v>14</v>
       </c>
+      <c r="H220">
+        <v>18</v>
+      </c>
+      <c r="I220">
+        <v>22</v>
+      </c>
       <c r="J220">
         <v>0</v>
       </c>
@@ -7536,6 +7566,12 @@
       <c r="G221" t="s">
         <v>15</v>
       </c>
+      <c r="H221">
+        <v>22</v>
+      </c>
+      <c r="I221">
+        <v>18</v>
+      </c>
       <c r="J221">
         <v>0</v>
       </c>
@@ -7562,6 +7598,12 @@
       <c r="G222" t="s">
         <v>15</v>
       </c>
+      <c r="H222">
+        <v>25</v>
+      </c>
+      <c r="I222">
+        <v>18</v>
+      </c>
       <c r="J222">
         <v>0</v>
       </c>
@@ -7588,6 +7630,12 @@
       <c r="G223" t="s">
         <v>14</v>
       </c>
+      <c r="H223">
+        <v>5</v>
+      </c>
+      <c r="I223">
+        <v>9</v>
+      </c>
       <c r="J223">
         <v>0</v>
       </c>
@@ -7614,6 +7662,12 @@
       <c r="G224" t="s">
         <v>15</v>
       </c>
+      <c r="H224">
+        <v>20</v>
+      </c>
+      <c r="I224">
+        <v>12</v>
+      </c>
       <c r="J224">
         <v>0</v>
       </c>
@@ -7640,6 +7694,12 @@
       <c r="G225" t="s">
         <v>15</v>
       </c>
+      <c r="H225">
+        <v>19</v>
+      </c>
+      <c r="I225">
+        <v>13</v>
+      </c>
       <c r="J225">
         <v>0</v>
       </c>
@@ -7666,6 +7726,12 @@
       <c r="G226" t="s">
         <v>15</v>
       </c>
+      <c r="H226">
+        <v>21</v>
+      </c>
+      <c r="I226">
+        <v>15</v>
+      </c>
       <c r="J226">
         <v>0</v>
       </c>
@@ -7692,6 +7758,12 @@
       <c r="G227" t="s">
         <v>14</v>
       </c>
+      <c r="H227">
+        <v>22</v>
+      </c>
+      <c r="I227">
+        <v>28</v>
+      </c>
       <c r="J227">
         <v>0</v>
       </c>
@@ -7718,6 +7790,12 @@
       <c r="G228" t="s">
         <v>15</v>
       </c>
+      <c r="H228">
+        <v>28</v>
+      </c>
+      <c r="I228">
+        <v>22</v>
+      </c>
       <c r="J228">
         <v>0</v>
       </c>
@@ -7744,6 +7822,12 @@
       <c r="G229" t="s">
         <v>14</v>
       </c>
+      <c r="H229">
+        <v>13</v>
+      </c>
+      <c r="I229">
+        <v>19</v>
+      </c>
       <c r="J229">
         <v>0</v>
       </c>
@@ -7770,6 +7854,12 @@
       <c r="G230" t="s">
         <v>15</v>
       </c>
+      <c r="H230">
+        <v>15</v>
+      </c>
+      <c r="I230">
+        <v>16</v>
+      </c>
       <c r="J230">
         <v>0</v>
       </c>
@@ -7796,6 +7886,12 @@
       <c r="G231" t="s">
         <v>14</v>
       </c>
+      <c r="H231">
+        <v>15</v>
+      </c>
+      <c r="I231">
+        <v>21</v>
+      </c>
       <c r="J231">
         <v>0</v>
       </c>
@@ -7822,6 +7918,12 @@
       <c r="G232" t="s">
         <v>14</v>
       </c>
+      <c r="H232">
+        <v>16</v>
+      </c>
+      <c r="I232">
+        <v>15</v>
+      </c>
       <c r="J232">
         <v>0</v>
       </c>
@@ -7848,6 +7950,12 @@
       <c r="G233" t="s">
         <v>15</v>
       </c>
+      <c r="H233">
+        <v>41</v>
+      </c>
+      <c r="I233">
+        <v>34</v>
+      </c>
       <c r="J233">
         <v>0</v>
       </c>
@@ -7874,6 +7982,12 @@
       <c r="G234" t="s">
         <v>14</v>
       </c>
+      <c r="H234">
+        <v>34</v>
+      </c>
+      <c r="I234">
+        <v>41</v>
+      </c>
       <c r="J234">
         <v>0</v>
       </c>
@@ -7900,6 +8014,12 @@
       <c r="G235" t="s">
         <v>14</v>
       </c>
+      <c r="H235">
+        <v>22</v>
+      </c>
+      <c r="I235">
+        <v>26</v>
+      </c>
       <c r="J235">
         <v>0</v>
       </c>
@@ -7926,6 +8046,12 @@
       <c r="G236" t="s">
         <v>15</v>
       </c>
+      <c r="H236">
+        <v>9</v>
+      </c>
+      <c r="I236">
+        <v>5</v>
+      </c>
       <c r="J236">
         <v>0</v>
       </c>
@@ -7952,6 +8078,12 @@
       <c r="G237" t="s">
         <v>14</v>
       </c>
+      <c r="H237">
+        <v>24</v>
+      </c>
+      <c r="I237">
+        <v>26</v>
+      </c>
       <c r="J237">
         <v>0</v>
       </c>
@@ -7978,6 +8110,12 @@
       <c r="G238" t="s">
         <v>15</v>
       </c>
+      <c r="H238">
+        <v>26</v>
+      </c>
+      <c r="I238">
+        <v>24</v>
+      </c>
       <c r="J238">
         <v>0</v>
       </c>
@@ -8004,6 +8142,12 @@
       <c r="G239" t="s">
         <v>15</v>
       </c>
+      <c r="H239">
+        <v>24</v>
+      </c>
+      <c r="I239">
+        <v>17</v>
+      </c>
       <c r="J239">
         <v>0</v>
       </c>
@@ -8030,6 +8174,12 @@
       <c r="G240" t="s">
         <v>14</v>
       </c>
+      <c r="H240">
+        <v>18</v>
+      </c>
+      <c r="I240">
+        <v>25</v>
+      </c>
       <c r="J240">
         <v>0</v>
       </c>
@@ -8056,6 +8206,12 @@
       <c r="G241" t="s">
         <v>15</v>
       </c>
+      <c r="H241">
+        <v>26</v>
+      </c>
+      <c r="I241">
+        <v>22</v>
+      </c>
       <c r="J241">
         <v>0</v>
       </c>
@@ -8082,6 +8238,12 @@
       <c r="G242" t="s">
         <v>14</v>
       </c>
+      <c r="H242">
+        <v>30</v>
+      </c>
+      <c r="I242">
+        <v>35</v>
+      </c>
       <c r="J242">
         <v>0</v>
       </c>
@@ -8107,6 +8269,12 @@
       </c>
       <c r="G243" t="s">
         <v>15</v>
+      </c>
+      <c r="H243">
+        <v>35</v>
+      </c>
+      <c r="I243">
+        <v>30</v>
       </c>
       <c r="J243">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 9 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B403FC79-FD4F-476A-8C20-1CC885C2C36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD784C83-6E99-4533-AB52-21A577FCA75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8302,6 +8302,12 @@
       <c r="G244" t="s">
         <v>15</v>
       </c>
+      <c r="H244">
+        <v>13</v>
+      </c>
+      <c r="I244">
+        <v>21</v>
+      </c>
       <c r="J244">
         <v>0</v>
       </c>
@@ -8328,6 +8334,12 @@
       <c r="G245" t="s">
         <v>14</v>
       </c>
+      <c r="H245">
+        <v>21</v>
+      </c>
+      <c r="I245">
+        <v>13</v>
+      </c>
       <c r="J245">
         <v>0</v>
       </c>
@@ -8354,6 +8366,12 @@
       <c r="G246" t="s">
         <v>14</v>
       </c>
+      <c r="H246">
+        <v>15</v>
+      </c>
+      <c r="I246">
+        <v>21</v>
+      </c>
       <c r="J246">
         <v>0</v>
       </c>
@@ -8380,6 +8398,12 @@
       <c r="G247" t="s">
         <v>15</v>
       </c>
+      <c r="H247">
+        <v>16</v>
+      </c>
+      <c r="I247">
+        <v>27</v>
+      </c>
       <c r="J247">
         <v>0</v>
       </c>
@@ -8406,6 +8430,12 @@
       <c r="G248" t="s">
         <v>15</v>
       </c>
+      <c r="H248">
+        <v>12</v>
+      </c>
+      <c r="I248">
+        <v>11</v>
+      </c>
       <c r="J248">
         <v>0</v>
       </c>
@@ -8432,6 +8462,12 @@
       <c r="G249" t="s">
         <v>15</v>
       </c>
+      <c r="H249">
+        <v>31</v>
+      </c>
+      <c r="I249">
+        <v>27</v>
+      </c>
       <c r="J249">
         <v>0</v>
       </c>
@@ -8458,6 +8494,12 @@
       <c r="G250" t="s">
         <v>14</v>
       </c>
+      <c r="H250">
+        <v>27</v>
+      </c>
+      <c r="I250">
+        <v>16</v>
+      </c>
       <c r="J250">
         <v>0</v>
       </c>
@@ -8484,6 +8526,12 @@
       <c r="G251" t="s">
         <v>14</v>
       </c>
+      <c r="H251">
+        <v>7</v>
+      </c>
+      <c r="I251">
+        <v>10</v>
+      </c>
       <c r="J251">
         <v>0</v>
       </c>
@@ -8510,6 +8558,12 @@
       <c r="G252" t="s">
         <v>14</v>
       </c>
+      <c r="H252">
+        <v>32</v>
+      </c>
+      <c r="I252">
+        <v>27</v>
+      </c>
       <c r="J252">
         <v>0</v>
       </c>
@@ -8536,6 +8590,12 @@
       <c r="G253" t="s">
         <v>14</v>
       </c>
+      <c r="H253">
+        <v>11</v>
+      </c>
+      <c r="I253">
+        <v>12</v>
+      </c>
       <c r="J253">
         <v>0</v>
       </c>
@@ -8562,6 +8622,12 @@
       <c r="G254" t="s">
         <v>14</v>
       </c>
+      <c r="H254">
+        <v>38</v>
+      </c>
+      <c r="I254">
+        <v>26</v>
+      </c>
       <c r="J254">
         <v>0</v>
       </c>
@@ -8588,6 +8654,12 @@
       <c r="G255" t="s">
         <v>14</v>
       </c>
+      <c r="H255">
+        <v>24</v>
+      </c>
+      <c r="I255">
+        <v>25</v>
+      </c>
       <c r="J255">
         <v>0</v>
       </c>
@@ -8614,6 +8686,12 @@
       <c r="G256" t="s">
         <v>14</v>
       </c>
+      <c r="H256">
+        <v>17</v>
+      </c>
+      <c r="I256">
+        <v>28</v>
+      </c>
       <c r="J256">
         <v>0</v>
       </c>
@@ -8640,6 +8718,12 @@
       <c r="G257" t="s">
         <v>15</v>
       </c>
+      <c r="H257">
+        <v>27</v>
+      </c>
+      <c r="I257">
+        <v>32</v>
+      </c>
       <c r="J257">
         <v>0</v>
       </c>
@@ -8666,6 +8750,12 @@
       <c r="G258" t="s">
         <v>15</v>
       </c>
+      <c r="H258">
+        <v>39</v>
+      </c>
+      <c r="I258">
+        <v>26</v>
+      </c>
       <c r="J258">
         <v>0</v>
       </c>
@@ -8692,6 +8782,12 @@
       <c r="G259" t="s">
         <v>15</v>
       </c>
+      <c r="H259">
+        <v>26</v>
+      </c>
+      <c r="I259">
+        <v>38</v>
+      </c>
       <c r="J259">
         <v>0</v>
       </c>
@@ -8718,6 +8814,12 @@
       <c r="G260" t="s">
         <v>15</v>
       </c>
+      <c r="H260">
+        <v>25</v>
+      </c>
+      <c r="I260">
+        <v>24</v>
+      </c>
       <c r="J260">
         <v>0</v>
       </c>
@@ -8744,6 +8846,12 @@
       <c r="G261" t="s">
         <v>15</v>
       </c>
+      <c r="H261">
+        <v>10</v>
+      </c>
+      <c r="I261">
+        <v>7</v>
+      </c>
       <c r="J261">
         <v>0</v>
       </c>
@@ -8770,6 +8878,12 @@
       <c r="G262" t="s">
         <v>14</v>
       </c>
+      <c r="H262">
+        <v>20</v>
+      </c>
+      <c r="I262">
+        <v>22</v>
+      </c>
       <c r="J262">
         <v>0</v>
       </c>
@@ -8796,6 +8910,12 @@
       <c r="G263" t="s">
         <v>14</v>
       </c>
+      <c r="H263">
+        <v>26</v>
+      </c>
+      <c r="I263">
+        <v>39</v>
+      </c>
       <c r="J263">
         <v>0</v>
       </c>
@@ -8822,6 +8942,12 @@
       <c r="G264" t="s">
         <v>14</v>
       </c>
+      <c r="H264">
+        <v>18</v>
+      </c>
+      <c r="I264">
+        <v>27</v>
+      </c>
       <c r="J264">
         <v>0</v>
       </c>
@@ -8848,6 +8974,12 @@
       <c r="G265" t="s">
         <v>15</v>
       </c>
+      <c r="H265">
+        <v>22</v>
+      </c>
+      <c r="I265">
+        <v>20</v>
+      </c>
       <c r="J265">
         <v>0</v>
       </c>
@@ -8874,6 +9006,12 @@
       <c r="G266" t="s">
         <v>15</v>
       </c>
+      <c r="H266">
+        <v>28</v>
+      </c>
+      <c r="I266">
+        <v>17</v>
+      </c>
       <c r="J266">
         <v>0</v>
       </c>
@@ -8900,6 +9038,12 @@
       <c r="G267" t="s">
         <v>15</v>
       </c>
+      <c r="H267">
+        <v>21</v>
+      </c>
+      <c r="I267">
+        <v>15</v>
+      </c>
       <c r="J267">
         <v>0</v>
       </c>
@@ -8926,6 +9070,12 @@
       <c r="G268" t="s">
         <v>15</v>
       </c>
+      <c r="H268">
+        <v>27</v>
+      </c>
+      <c r="I268">
+        <v>18</v>
+      </c>
       <c r="J268">
         <v>0</v>
       </c>
@@ -8952,6 +9102,12 @@
       <c r="G269" t="s">
         <v>14</v>
       </c>
+      <c r="H269">
+        <v>35</v>
+      </c>
+      <c r="I269">
+        <v>30</v>
+      </c>
       <c r="J269">
         <v>0</v>
       </c>
@@ -8978,6 +9134,12 @@
       <c r="G270" t="s">
         <v>14</v>
       </c>
+      <c r="H270">
+        <v>27</v>
+      </c>
+      <c r="I270">
+        <v>31</v>
+      </c>
       <c r="J270">
         <v>0</v>
       </c>
@@ -9004,6 +9166,12 @@
       <c r="G271" t="s">
         <v>15</v>
       </c>
+      <c r="H271">
+        <v>30</v>
+      </c>
+      <c r="I271">
+        <v>35</v>
+      </c>
       <c r="J271">
         <v>0</v>
       </c>
@@ -9030,8 +9198,14 @@
       <c r="G272" t="s">
         <v>14</v>
       </c>
+      <c r="H272">
+        <v>16</v>
+      </c>
+      <c r="I272">
+        <v>13</v>
+      </c>
       <c r="J272">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.35">
@@ -9056,8 +9230,14 @@
       <c r="G273" t="s">
         <v>15</v>
       </c>
+      <c r="H273">
+        <v>13</v>
+      </c>
+      <c r="I273">
+        <v>16</v>
+      </c>
       <c r="J273">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add Week 11 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BEDE23-F2A5-4062-8928-EDF60046957F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED904D42-EA40-443C-8072-FD5EAC560BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10158,6 +10158,12 @@
       <c r="G302" t="s">
         <v>15</v>
       </c>
+      <c r="H302">
+        <v>25</v>
+      </c>
+      <c r="I302">
+        <v>16</v>
+      </c>
       <c r="J302">
         <v>0</v>
       </c>
@@ -10184,6 +10190,12 @@
       <c r="G303" t="s">
         <v>14</v>
       </c>
+      <c r="H303">
+        <v>16</v>
+      </c>
+      <c r="I303">
+        <v>25</v>
+      </c>
       <c r="J303">
         <v>0</v>
       </c>
@@ -10210,6 +10222,12 @@
       <c r="G304" t="s">
         <v>14</v>
       </c>
+      <c r="H304">
+        <v>17</v>
+      </c>
+      <c r="I304">
+        <v>31</v>
+      </c>
       <c r="J304">
         <v>0</v>
       </c>
@@ -10236,6 +10254,12 @@
       <c r="G305" t="s">
         <v>14</v>
       </c>
+      <c r="H305">
+        <v>24</v>
+      </c>
+      <c r="I305">
+        <v>14</v>
+      </c>
       <c r="J305">
         <v>0</v>
       </c>
@@ -10262,6 +10286,12 @@
       <c r="G306" t="s">
         <v>15</v>
       </c>
+      <c r="H306">
+        <v>56</v>
+      </c>
+      <c r="I306">
+        <v>34</v>
+      </c>
       <c r="J306">
         <v>0</v>
       </c>
@@ -10288,6 +10318,12 @@
       <c r="G307" t="s">
         <v>15</v>
       </c>
+      <c r="H307">
+        <v>14</v>
+      </c>
+      <c r="I307">
+        <v>24</v>
+      </c>
       <c r="J307">
         <v>0</v>
       </c>
@@ -10314,6 +10350,12 @@
       <c r="G308" t="s">
         <v>15</v>
       </c>
+      <c r="H308">
+        <v>34</v>
+      </c>
+      <c r="I308">
+        <v>27</v>
+      </c>
       <c r="J308">
         <v>0</v>
       </c>
@@ -10340,6 +10382,12 @@
       <c r="G309" t="s">
         <v>15</v>
       </c>
+      <c r="H309">
+        <v>32</v>
+      </c>
+      <c r="I309">
+        <v>24</v>
+      </c>
       <c r="J309">
         <v>0</v>
       </c>
@@ -10366,6 +10414,12 @@
       <c r="G310" t="s">
         <v>15</v>
       </c>
+      <c r="H310">
+        <v>3</v>
+      </c>
+      <c r="I310">
+        <v>8</v>
+      </c>
       <c r="J310">
         <v>0</v>
       </c>
@@ -10392,6 +10446,12 @@
       <c r="G311" t="s">
         <v>15</v>
       </c>
+      <c r="H311">
+        <v>38</v>
+      </c>
+      <c r="I311">
+        <v>26</v>
+      </c>
       <c r="J311">
         <v>0</v>
       </c>
@@ -10418,6 +10478,12 @@
       <c r="G312" t="s">
         <v>14</v>
       </c>
+      <c r="H312">
+        <v>26</v>
+      </c>
+      <c r="I312">
+        <v>23</v>
+      </c>
       <c r="J312">
         <v>0</v>
       </c>
@@ -10444,6 +10510,12 @@
       <c r="G313" t="s">
         <v>15</v>
       </c>
+      <c r="H313">
+        <v>31</v>
+      </c>
+      <c r="I313">
+        <v>17</v>
+      </c>
       <c r="J313">
         <v>0</v>
       </c>
@@ -10470,6 +10542,12 @@
       <c r="G314" t="s">
         <v>14</v>
       </c>
+      <c r="H314">
+        <v>34</v>
+      </c>
+      <c r="I314">
+        <v>56</v>
+      </c>
       <c r="J314">
         <v>0</v>
       </c>
@@ -10496,6 +10574,12 @@
       <c r="G315" t="s">
         <v>14</v>
       </c>
+      <c r="H315">
+        <v>17</v>
+      </c>
+      <c r="I315">
+        <v>30</v>
+      </c>
       <c r="J315">
         <v>0</v>
       </c>
@@ -10522,6 +10606,12 @@
       <c r="G316" t="s">
         <v>14</v>
       </c>
+      <c r="H316">
+        <v>27</v>
+      </c>
+      <c r="I316">
+        <v>34</v>
+      </c>
       <c r="J316">
         <v>0</v>
       </c>
@@ -10548,6 +10638,12 @@
       <c r="G317" t="s">
         <v>15</v>
       </c>
+      <c r="H317">
+        <v>23</v>
+      </c>
+      <c r="I317">
+        <v>26</v>
+      </c>
       <c r="J317">
         <v>0</v>
       </c>
@@ -10574,6 +10670,12 @@
       <c r="G318" t="s">
         <v>14</v>
       </c>
+      <c r="H318">
+        <v>21</v>
+      </c>
+      <c r="I318">
+        <v>35</v>
+      </c>
       <c r="J318">
         <v>0</v>
       </c>
@@ -10600,6 +10702,12 @@
       <c r="G319" t="s">
         <v>14</v>
       </c>
+      <c r="H319">
+        <v>8</v>
+      </c>
+      <c r="I319">
+        <v>3</v>
+      </c>
       <c r="J319">
         <v>0</v>
       </c>
@@ -10626,6 +10734,12 @@
       <c r="G320" t="s">
         <v>15</v>
       </c>
+      <c r="H320">
+        <v>21</v>
+      </c>
+      <c r="I320">
+        <v>12</v>
+      </c>
       <c r="J320">
         <v>0</v>
       </c>
@@ -10652,6 +10766,12 @@
       <c r="G321" t="s">
         <v>14</v>
       </c>
+      <c r="H321">
+        <v>12</v>
+      </c>
+      <c r="I321">
+        <v>21</v>
+      </c>
       <c r="J321">
         <v>0</v>
       </c>
@@ -10678,6 +10798,12 @@
       <c r="G322" t="s">
         <v>15</v>
       </c>
+      <c r="H322">
+        <v>35</v>
+      </c>
+      <c r="I322">
+        <v>21</v>
+      </c>
       <c r="J322">
         <v>0</v>
       </c>
@@ -10704,6 +10830,12 @@
       <c r="G323" t="s">
         <v>15</v>
       </c>
+      <c r="H323">
+        <v>30</v>
+      </c>
+      <c r="I323">
+        <v>17</v>
+      </c>
       <c r="J323">
         <v>0</v>
       </c>
@@ -10730,6 +10862,12 @@
       <c r="G324" t="s">
         <v>14</v>
       </c>
+      <c r="H324">
+        <v>26</v>
+      </c>
+      <c r="I324">
+        <v>38</v>
+      </c>
       <c r="J324">
         <v>0</v>
       </c>
@@ -10756,6 +10894,12 @@
       <c r="G325" t="s">
         <v>14</v>
       </c>
+      <c r="H325">
+        <v>24</v>
+      </c>
+      <c r="I325">
+        <v>32</v>
+      </c>
       <c r="J325">
         <v>0</v>
       </c>
@@ -10782,6 +10926,12 @@
       <c r="G326" t="s">
         <v>14</v>
       </c>
+      <c r="H326">
+        <v>11</v>
+      </c>
+      <c r="I326">
+        <v>18</v>
+      </c>
       <c r="J326">
         <v>0</v>
       </c>
@@ -10807,6 +10957,12 @@
       </c>
       <c r="G327" t="s">
         <v>15</v>
+      </c>
+      <c r="H327">
+        <v>18</v>
+      </c>
+      <c r="I327">
+        <v>11</v>
       </c>
       <c r="J327">
         <v>0</v>

</xml_diff>

<commit_message>
Add Week 12 (Tester) results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED904D42-EA40-443C-8072-FD5EAC560BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{158B873D-BE89-4716-8092-9C869E8C8FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10990,6 +10990,12 @@
       <c r="G328" t="s">
         <v>14</v>
       </c>
+      <c r="H328">
+        <v>30</v>
+      </c>
+      <c r="I328">
+        <v>33</v>
+      </c>
       <c r="J328">
         <v>0</v>
       </c>
@@ -11016,6 +11022,12 @@
       <c r="G329" t="s">
         <v>15</v>
       </c>
+      <c r="H329">
+        <v>33</v>
+      </c>
+      <c r="I329">
+        <v>30</v>
+      </c>
       <c r="J329">
         <v>0</v>
       </c>
@@ -11042,6 +11054,12 @@
       <c r="G330" t="s">
         <v>15</v>
       </c>
+      <c r="H330">
+        <v>38</v>
+      </c>
+      <c r="I330">
+        <v>34</v>
+      </c>
       <c r="J330">
         <v>0</v>
       </c>
@@ -11068,6 +11086,12 @@
       <c r="G331" t="s">
         <v>14</v>
       </c>
+      <c r="H331">
+        <v>33</v>
+      </c>
+      <c r="I331">
+        <v>26</v>
+      </c>
       <c r="J331">
         <v>0</v>
       </c>
@@ -11094,6 +11118,12 @@
       <c r="G332" t="s">
         <v>15</v>
       </c>
+      <c r="H332">
+        <v>29</v>
+      </c>
+      <c r="I332">
+        <v>27</v>
+      </c>
       <c r="J332">
         <v>0</v>
       </c>
@@ -11120,6 +11150,12 @@
       <c r="G333" t="s">
         <v>15</v>
       </c>
+      <c r="H333">
+        <v>26</v>
+      </c>
+      <c r="I333">
+        <v>33</v>
+      </c>
       <c r="J333">
         <v>0</v>
       </c>
@@ -11146,6 +11182,12 @@
       <c r="G334" t="s">
         <v>14</v>
       </c>
+      <c r="H334">
+        <v>34</v>
+      </c>
+      <c r="I334">
+        <v>38</v>
+      </c>
       <c r="J334">
         <v>0</v>
       </c>
@@ -11172,6 +11214,12 @@
       <c r="G335" t="s">
         <v>14</v>
       </c>
+      <c r="H335">
+        <v>27</v>
+      </c>
+      <c r="I335">
+        <v>29</v>
+      </c>
       <c r="J335">
         <v>0</v>
       </c>
@@ -11198,6 +11246,12 @@
       <c r="G336" t="s">
         <v>14</v>
       </c>
+      <c r="H336">
+        <v>2</v>
+      </c>
+      <c r="I336">
+        <v>4</v>
+      </c>
       <c r="J336">
         <v>0</v>
       </c>
@@ -11224,6 +11278,12 @@
       <c r="G337" t="s">
         <v>15</v>
       </c>
+      <c r="H337">
+        <v>4</v>
+      </c>
+      <c r="I337">
+        <v>2</v>
+      </c>
       <c r="J337">
         <v>0</v>
       </c>
@@ -11250,6 +11310,12 @@
       <c r="G338" t="s">
         <v>15</v>
       </c>
+      <c r="H338">
+        <v>22</v>
+      </c>
+      <c r="I338">
+        <v>18</v>
+      </c>
       <c r="J338">
         <v>0</v>
       </c>
@@ -11276,6 +11342,12 @@
       <c r="G339" t="s">
         <v>14</v>
       </c>
+      <c r="H339">
+        <v>20</v>
+      </c>
+      <c r="I339">
+        <v>21</v>
+      </c>
       <c r="J339">
         <v>0</v>
       </c>
@@ -11302,6 +11374,12 @@
       <c r="G340" t="s">
         <v>14</v>
       </c>
+      <c r="H340">
+        <v>20</v>
+      </c>
+      <c r="I340">
+        <v>22</v>
+      </c>
       <c r="J340">
         <v>0</v>
       </c>
@@ -11328,6 +11406,12 @@
       <c r="G341" t="s">
         <v>15</v>
       </c>
+      <c r="H341">
+        <v>36</v>
+      </c>
+      <c r="I341">
+        <v>25</v>
+      </c>
       <c r="J341">
         <v>0</v>
       </c>
@@ -11354,6 +11438,12 @@
       <c r="G342" t="s">
         <v>15</v>
       </c>
+      <c r="H342">
+        <v>5</v>
+      </c>
+      <c r="I342">
+        <v>11</v>
+      </c>
       <c r="J342">
         <v>0</v>
       </c>
@@ -11380,6 +11470,12 @@
       <c r="G343" t="s">
         <v>15</v>
       </c>
+      <c r="H343">
+        <v>22</v>
+      </c>
+      <c r="I343">
+        <v>20</v>
+      </c>
       <c r="J343">
         <v>0</v>
       </c>
@@ -11406,6 +11502,12 @@
       <c r="G344" t="s">
         <v>15</v>
       </c>
+      <c r="H344">
+        <v>19</v>
+      </c>
+      <c r="I344">
+        <v>22</v>
+      </c>
       <c r="J344">
         <v>0</v>
       </c>
@@ -11432,6 +11534,12 @@
       <c r="G345" t="s">
         <v>15</v>
       </c>
+      <c r="H345">
+        <v>13</v>
+      </c>
+      <c r="I345">
+        <v>14</v>
+      </c>
       <c r="J345">
         <v>0</v>
       </c>
@@ -11458,8 +11566,14 @@
       <c r="G346" t="s">
         <v>15</v>
       </c>
+      <c r="H346">
+        <v>14</v>
+      </c>
+      <c r="I346">
+        <v>14</v>
+      </c>
       <c r="J346">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.35">
@@ -11484,6 +11598,12 @@
       <c r="G347" t="s">
         <v>15</v>
       </c>
+      <c r="H347">
+        <v>21</v>
+      </c>
+      <c r="I347">
+        <v>20</v>
+      </c>
       <c r="J347">
         <v>0</v>
       </c>
@@ -11510,6 +11630,12 @@
       <c r="G348" t="s">
         <v>14</v>
       </c>
+      <c r="H348">
+        <v>26</v>
+      </c>
+      <c r="I348">
+        <v>22</v>
+      </c>
       <c r="J348">
         <v>0</v>
       </c>
@@ -11536,6 +11662,12 @@
       <c r="G349" t="s">
         <v>14</v>
       </c>
+      <c r="H349">
+        <v>25</v>
+      </c>
+      <c r="I349">
+        <v>36</v>
+      </c>
       <c r="J349">
         <v>0</v>
       </c>
@@ -11562,6 +11694,12 @@
       <c r="G350" t="s">
         <v>14</v>
       </c>
+      <c r="H350">
+        <v>22</v>
+      </c>
+      <c r="I350">
+        <v>19</v>
+      </c>
       <c r="J350">
         <v>0</v>
       </c>
@@ -11588,8 +11726,14 @@
       <c r="G351" t="s">
         <v>14</v>
       </c>
+      <c r="H351">
+        <v>14</v>
+      </c>
+      <c r="I351">
+        <v>14</v>
+      </c>
       <c r="J351">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.35">
@@ -11614,6 +11758,12 @@
       <c r="G352" t="s">
         <v>14</v>
       </c>
+      <c r="H352">
+        <v>11</v>
+      </c>
+      <c r="I352">
+        <v>5</v>
+      </c>
       <c r="J352">
         <v>0</v>
       </c>
@@ -11640,6 +11790,12 @@
       <c r="G353" t="s">
         <v>15</v>
       </c>
+      <c r="H353">
+        <v>22</v>
+      </c>
+      <c r="I353">
+        <v>26</v>
+      </c>
       <c r="J353">
         <v>0</v>
       </c>
@@ -11666,6 +11822,12 @@
       <c r="G354" t="s">
         <v>14</v>
       </c>
+      <c r="H354">
+        <v>14</v>
+      </c>
+      <c r="I354">
+        <v>16</v>
+      </c>
       <c r="J354">
         <v>0</v>
       </c>
@@ -11692,6 +11854,12 @@
       <c r="G355" t="s">
         <v>15</v>
       </c>
+      <c r="H355">
+        <v>16</v>
+      </c>
+      <c r="I355">
+        <v>14</v>
+      </c>
       <c r="J355">
         <v>0</v>
       </c>
@@ -11718,6 +11886,12 @@
       <c r="G356" t="s">
         <v>14</v>
       </c>
+      <c r="H356">
+        <v>14</v>
+      </c>
+      <c r="I356">
+        <v>13</v>
+      </c>
       <c r="J356">
         <v>0</v>
       </c>
@@ -11744,6 +11918,12 @@
       <c r="G357" t="s">
         <v>14</v>
       </c>
+      <c r="H357">
+        <v>18</v>
+      </c>
+      <c r="I357">
+        <v>22</v>
+      </c>
       <c r="J357">
         <v>0</v>
       </c>
@@ -11770,6 +11950,12 @@
       <c r="G358" t="s">
         <v>14</v>
       </c>
+      <c r="H358">
+        <v>10</v>
+      </c>
+      <c r="I358">
+        <v>22</v>
+      </c>
       <c r="J358">
         <v>0</v>
       </c>
@@ -11795,6 +11981,12 @@
       </c>
       <c r="G359" t="s">
         <v>15</v>
+      </c>
+      <c r="H359">
+        <v>22</v>
+      </c>
+      <c r="I359">
+        <v>10</v>
       </c>
       <c r="J359">
         <v>0</v>

</xml_diff>